<commit_message>
update on 2025 human review
</commit_message>
<xml_diff>
--- a/human_adjudication/human_adjudication_v_2_4_1/2025/human_adjudication_v_2_4_1_2025_R_B.xlsx
+++ b/human_adjudication/human_adjudication_v_2_4_1/2025/human_adjudication_v_2_4_1_2025_R_B.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\bulun-debian\ai-paper-val\human_adjudication\human_adjudication_v_2_4_1\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{285DAA0F-5730-4B8B-9779-1FFEF4FFB832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B834C5-6C0B-4E1D-A8D5-DF7652FE51A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="967" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="967" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1301" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1369" uniqueCount="644">
   <si>
     <t>Field</t>
   </si>
@@ -2021,6 +2021,66 @@
   </si>
   <si>
     <t>C006 identifies a discrepancy in the stated confidence-interval method. Although the supplementary materials describe several low-event-count results as using exact 95% confidence intervals, the reported intervals are reproducible as log-Wald approximate intervals.</t>
+  </si>
+  <si>
+    <t>Compared with the original protocol, the primary composite endpoint reported in the paper incorporated an additional HbA1c failure criterion. Participants were classified as not having achieved the primary endpoint if their HbA1c was ≥6.5% at either the 6- or 12-month assessment, regardless of whether they had met the prespecified weight-loss or physical-activity target.</t>
+  </si>
+  <si>
+    <t>eTable 16 (Supp2 p.59) MI-pooled risks 32.2% (AI) vs 31.9% (human) imply RD +0.3 points, but RD is printed -1.1 (one-sided bound -11.5). With Rubin's rules and the unadjusted RD model, pooled RD equals the difference of pooled risks.</t>
+  </si>
+  <si>
+    <t>Protocol (Supp1 pp.6, 15; OCR) averages PA over months 6-11 for the weight-plus-PA branch; Supp2 p.13 averages weekly MVPA over all post-baseline visits (max 11; eTable 8b months 1-11). Amendment v1.4 (03-28-2022; Supp1 p.80) says the PA time frame was 'clarified' but the revised window is not printed, so whether the report follows the amended window cannot be determined.</t>
+  </si>
+  <si>
+    <t>eTable 6 footnote (Supp2 p.45) gives site P=.024 and ethnicity P=.018; from the printed counts (p.44) site gives P=.063 (chi-square), .082 (Yates), .070 (Fisher); ethnicity .064 (chi-square, 4 categories), .055 (Fisher), .035-.044 (2 categories). Neither printed P reproduces.</t>
+  </si>
+  <si>
+    <t>Restriction of the HbA1c-reduction branch to baseline HbA1c 5.7-6.4% was made by dated protocol amendment v1.4 (03-28-2022; Supp1 pp.80-81, OCR), and the report (main p.3; Figure 2 footnote c, 130/130) follows the amended protocol. No difference between the report and the operative plan.</t>
+  </si>
+  <si>
+    <t>eTable 1b (Supp2 p.37): versions 11.100.131 and 122.100.407 each show 5 (5%) of the 183 AI participants; 5/183=2.7%. The other seven rows reproduce with N=183 (e.g., 58/183=31.7%-&gt;32; 109/183=59.6%-&gt;60).</t>
+  </si>
+  <si>
+    <t>The primary analysis was changed from the original protocol’s approach of excluding participants who withdrew or lacked 12-month data to an approach that included all randomized participants and classified those with missing 12-month outcome data as not having achieved the primary endpoint. This change affected both the analysis population and the method for handling missing outcome data. The participant counts reported in the paper are internally consistent.</t>
+  </si>
+  <si>
+    <t>Supp2 p.13: weekly MVPA from valid wear periods is summed and divided by the number of available periods (max 11); non-compliant weeks/months get 0 (pp.13, 30, 49). Summing valid periods (zeros add nothing) over all available periods is exactly zero-imputation, so the descriptions are compatible.</t>
+  </si>
+  <si>
+    <t>Protocol §9.4.7-9.4.8 (Supp1 p.38; OCR) analyzes the primary and component end points with (mixed-effects) logistic regression; report uses unadjusted binomial regression for the risk difference (main p.4). Disclosed in the SAP change table (Supp1 p.86); cluster-robust SEs added post hoc (eTables 19a-b).</t>
+  </si>
+  <si>
+    <t>Supp2 p.13 says missing data within valid days were interpolated and that the printed R code was used; in both loops (pp.15-16) ac_imp is computed but activity_stats() and BoutsOfPA() receive the raw vector ac, and the three BoutsOfPA calls are identical (no threshold argument), so threshold-specific bout outputs cannot differ. Since the missing rate is unkown, the potential impact and substantiveness is hard to determine.</t>
+  </si>
+  <si>
+    <t>Protocol §9.4.2/9.4.8 (Supp1 pp.38-39; OCR) plans multiple imputation for PA if &gt;5% missing, with a complete-case sensitivity analysis; report assigns 0 min/week to non-wear periods (worst case; Supp2 pp.13, 30, 49) with best-case sensitivity analyses. Disclosed in the SAP change table (Supp1 p.86).</t>
+  </si>
+  <si>
+    <t>Protocol §5.5.1/Table 1 (Supp1 p.18; OCR) recruitment-pool figures are inconsistent (21,410 vs 21,346 eligible; 13,910/21,346=65.2% printed 56%; 4,892/8,751=55.9% printed 60%), but these are feasibility estimates of portal access, not a design element the analysis relies on.</t>
+  </si>
+  <si>
+    <t>Under the original protocol, the per-protocol analysis was to be conducted in participants who completed the intervention program. In the report, however, the analysis population was redefined as participants with complete 12-month outcome data who had not initiated prohibited medications. The protocol-defined and report-defined populations therefore differed in both their inclusion criteria and sample sizes.</t>
+  </si>
+  <si>
+    <t>It is unclear from the descriptions provided in different sections of the paper whether the Fine–Gray model that yielded the primary endpoint estimate of sHR = 1.02 (95% CI, 0.74–1.39) included study center as a covariate.</t>
+  </si>
+  <si>
+    <t>SAP §3.6 (Supp2 pp.7-9, OCR) and protocol statistical sections plan etiology-adjusted Cox, general linear and Poisson models (with log-rank/Wilcoxon tests) for mortality, ECMO/ventilation/organ failure-free days, ICU/hospital stay and SAE counts; the report gives unadjusted differences with bootstrap CIs and crude RRs (Table 2 footnotes b-c), and no adjusted secondary output.</t>
+  </si>
+  <si>
+    <t>C002 concerns the SOFA component threshold used to define “organ failure/free days.” The SAP specified organ failure as a score &gt;2 in at least one SOFA component, whereas the main article required every component score to be 0 or 1 for a day to qualify as free of organ failure. These definitions differ in how they classify days on which a component score is exactly 2.</t>
+  </si>
+  <si>
+    <t>The protocol specified a post–cardiac arrest subgroup; however, the paper described a broader “Other” subgroup as predefined or prespecified and reported results for that subgroup. No separate results for the post–cardiac arrest subgroup were identified in the materials provided.</t>
+  </si>
+  <si>
+    <t>Protocol (Supp1 pp.14-15 and repeats) and SAP §2.2/§3.6 (Supp2 pp.4, 7-8) plan ECMO-free and ventilation-free days at D30 and D60; main p.3 lists both windows as predefined, but only day-30 values are reported (Table 2 p.6; eTable 3 Supp3 p.5). Searched main and Supp3 for D60 free-day outputs: none. A narrative summary was provided (main paper page 7), but Day 60 (D60) free-day outcomes were not reported in a form that allowed them to be separately identified, extracted, and verified.</t>
+  </si>
+  <si>
+    <t>SAP §2.2/§3.6 (Supp2 pp.4, 7; OCR) define MACE without dialysis; the protocol (Supp1 pp.8, 14-15, all versions) and the report (main p.3; eTable 3 component rows, Supp3 p.5) include dialysis. The report is itself inconsistent: eFigure 4 title (Supp3 p.1/p.10) defines MACE without dialysis.</t>
+  </si>
+  <si>
+    <t>SAP §3.6 (Supp2 p.8, OCR) analyzes left ventricular function at day 30 with a Global Net Benefit hierarchical composite (death, heart transplant, LVEF &gt;30%) with bootstrap CI; the report gives only median LVEF among survivors, 45 vs 40%, difference 5 (-0 to 10) (eTable 3, Supp3 p.5). Protocol lists LVEF at day 30 without the composite.</t>
   </si>
 </sst>
 </file>
@@ -3115,16 +3175,18 @@
       <c r="C2" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D2" s="8"/>
+      <c r="D2" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E2" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G2" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A2="",COUNTIF($A$2:$A$14,A2)&lt;&gt;1,LEFT(A2,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D2="retain",E2="statistical_results")),H2&lt;&gt;"",NOT(EXACT(H2,"not_applicable"))),AND(NOT(AND(D2="retain",E2="statistical_results")),I2&lt;&gt;"",NOT(EXACT(I2,"not_applicable"))),AND(NOT(AND(D2="retain",E2="statistical_results")),J2&lt;&gt;"",NOT(EXACT(J2,"not_applicable"))),AND(NOT(AND(D2="retain",OR(E2="report_internal_inconsistency",E2="plan_material"))),K2&lt;&gt;"",NOT(EXACT(K2,"not_applicable"))),AND(NOT(AND(D2="retain",E2="protocol_report")),L2&lt;&gt;"",NOT(EXACT(L2,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D2,"retain"),EXACT(D2,"exclude"),EXACT(D2,"discuss"))),NOT(OR(EXACT(E2,"statistical_results"),EXACT(E2,"report_internal_inconsistency"),EXACT(E2,"plan_material"),EXACT(E2,"protocol_report"))),AND(AND(D2="retain",E2="statistical_results"),NOT(OR(EXACT(H2,"confirmed_issue"),EXACT(H2,"probable_issue"),EXACT(H2,"not_issue"),EXACT(H2,"indeterminate")))),AND(AND(D2="retain",E2="statistical_results"),NOT(OR(EXACT(I2,"substantive"),EXACT(I2,"minor_presentation"),EXACT(I2,"indeterminate")))),AND(AND(D2="retain",E2="statistical_results"),J2&lt;&gt;"",NOT(OR(EXACT(J2,"direct"),EXACT(J2,"possible"),EXACT(J2,"unlikely"),EXACT(J2,"unknown")))),AND(AND(D2="retain",OR(E2="report_internal_inconsistency",E2="plan_material")),NOT(OR(EXACT(K2,"substantive_inconsistency"),EXACT(K2,"minor_presentation"),EXACT(K2,"non_inconsistency"),EXACT(K2,"indeterminate")))),AND(AND(D2="retain",E2="protocol_report"),L2&lt;&gt;"",NOT(OR(EXACT(L2,"substantive_difference"),EXACT(L2,"minor_presentation"),EXACT(L2,"version_timing"),EXACT(L2,"non_inconsistency"),EXACT(L2,"indeterminate"))))),"CHECK FIELDS",IF(AND(F2&lt;&gt;"",NOT(OR(EXACT(F2,"no"),EXACT(F2,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F2,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H2" s="8" t="str">
         <f t="shared" ref="H2:H14" si="0">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
@@ -3142,16 +3204,17 @@
         <f t="shared" ref="K2:K14" si="3">IF(AND(OR(D2="retain",D2=""),OR(E2="report_internal_inconsistency",E2="plan_material")),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
-      <c r="L2" s="9" t="str">
-        <f t="shared" ref="L2:L14" si="4">IF(AND(OR(D2="retain",D2=""),E2="protocol_report"),"","not_applicable")</f>
-        <v/>
+      <c r="L2" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M2" s="3"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
-      <c r="R2" s="9"/>
+      <c r="R2" s="9" t="s">
+        <v>624</v>
+      </c>
     </row>
     <row r="3" spans="1:18" ht="91.95" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -3163,16 +3226,18 @@
       <c r="C3" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="D3" s="8"/>
+      <c r="D3" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E3" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G3" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A3="",COUNTIF($A$2:$A$14,A3)&lt;&gt;1,LEFT(A3,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D3="retain",E3="statistical_results")),H3&lt;&gt;"",NOT(EXACT(H3,"not_applicable"))),AND(NOT(AND(D3="retain",E3="statistical_results")),I3&lt;&gt;"",NOT(EXACT(I3,"not_applicable"))),AND(NOT(AND(D3="retain",E3="statistical_results")),J3&lt;&gt;"",NOT(EXACT(J3,"not_applicable"))),AND(NOT(AND(D3="retain",OR(E3="report_internal_inconsistency",E3="plan_material"))),K3&lt;&gt;"",NOT(EXACT(K3,"not_applicable"))),AND(NOT(AND(D3="retain",E3="protocol_report")),L3&lt;&gt;"",NOT(EXACT(L3,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D3,"retain"),EXACT(D3,"exclude"),EXACT(D3,"discuss"))),NOT(OR(EXACT(E3,"statistical_results"),EXACT(E3,"report_internal_inconsistency"),EXACT(E3,"plan_material"),EXACT(E3,"protocol_report"))),AND(AND(D3="retain",E3="statistical_results"),NOT(OR(EXACT(H3,"confirmed_issue"),EXACT(H3,"probable_issue"),EXACT(H3,"not_issue"),EXACT(H3,"indeterminate")))),AND(AND(D3="retain",E3="statistical_results"),NOT(OR(EXACT(I3,"substantive"),EXACT(I3,"minor_presentation"),EXACT(I3,"indeterminate")))),AND(AND(D3="retain",E3="statistical_results"),J3&lt;&gt;"",NOT(OR(EXACT(J3,"direct"),EXACT(J3,"possible"),EXACT(J3,"unlikely"),EXACT(J3,"unknown")))),AND(AND(D3="retain",OR(E3="report_internal_inconsistency",E3="plan_material")),NOT(OR(EXACT(K3,"substantive_inconsistency"),EXACT(K3,"minor_presentation"),EXACT(K3,"non_inconsistency"),EXACT(K3,"indeterminate")))),AND(AND(D3="retain",E3="protocol_report"),L3&lt;&gt;"",NOT(OR(EXACT(L3,"substantive_difference"),EXACT(L3,"minor_presentation"),EXACT(L3,"version_timing"),EXACT(L3,"non_inconsistency"),EXACT(L3,"indeterminate"))))),"CHECK FIELDS",IF(AND(F3&lt;&gt;"",NOT(OR(EXACT(F3,"no"),EXACT(F3,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F3,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H3" s="8" t="str">
         <f t="shared" si="0"/>
@@ -3190,16 +3255,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L3" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L3" s="9" t="s">
+        <v>557</v>
       </c>
       <c r="M3" s="1"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="9"/>
+      <c r="R3" s="9" t="s">
+        <v>626</v>
+      </c>
     </row>
     <row r="4" spans="1:18" ht="91.95" customHeight="1">
       <c r="A4" s="3" t="s">
@@ -3211,16 +3277,18 @@
       <c r="C4" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="D4" s="8"/>
+      <c r="D4" s="8" t="s">
+        <v>488</v>
+      </c>
       <c r="E4" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G4" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A4="",COUNTIF($A$2:$A$14,A4)&lt;&gt;1,LEFT(A4,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D4="retain",E4="statistical_results")),H4&lt;&gt;"",NOT(EXACT(H4,"not_applicable"))),AND(NOT(AND(D4="retain",E4="statistical_results")),I4&lt;&gt;"",NOT(EXACT(I4,"not_applicable"))),AND(NOT(AND(D4="retain",E4="statistical_results")),J4&lt;&gt;"",NOT(EXACT(J4,"not_applicable"))),AND(NOT(AND(D4="retain",OR(E4="report_internal_inconsistency",E4="plan_material"))),K4&lt;&gt;"",NOT(EXACT(K4,"not_applicable"))),AND(NOT(AND(D4="retain",E4="protocol_report")),L4&lt;&gt;"",NOT(EXACT(L4,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D4,"retain"),EXACT(D4,"exclude"),EXACT(D4,"discuss"))),NOT(OR(EXACT(E4,"statistical_results"),EXACT(E4,"report_internal_inconsistency"),EXACT(E4,"plan_material"),EXACT(E4,"protocol_report"))),AND(AND(D4="retain",E4="statistical_results"),NOT(OR(EXACT(H4,"confirmed_issue"),EXACT(H4,"probable_issue"),EXACT(H4,"not_issue"),EXACT(H4,"indeterminate")))),AND(AND(D4="retain",E4="statistical_results"),NOT(OR(EXACT(I4,"substantive"),EXACT(I4,"minor_presentation"),EXACT(I4,"indeterminate")))),AND(AND(D4="retain",E4="statistical_results"),J4&lt;&gt;"",NOT(OR(EXACT(J4,"direct"),EXACT(J4,"possible"),EXACT(J4,"unlikely"),EXACT(J4,"unknown")))),AND(AND(D4="retain",OR(E4="report_internal_inconsistency",E4="plan_material")),NOT(OR(EXACT(K4,"substantive_inconsistency"),EXACT(K4,"minor_presentation"),EXACT(K4,"non_inconsistency"),EXACT(K4,"indeterminate")))),AND(AND(D4="retain",E4="protocol_report"),L4&lt;&gt;"",NOT(OR(EXACT(L4,"substantive_difference"),EXACT(L4,"minor_presentation"),EXACT(L4,"version_timing"),EXACT(L4,"non_inconsistency"),EXACT(L4,"indeterminate"))))),"CHECK FIELDS",IF(AND(F4&lt;&gt;"",NOT(OR(EXACT(F4,"no"),EXACT(F4,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F4,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H4" s="8" t="str">
         <f t="shared" si="0"/>
@@ -3238,16 +3306,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L4" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L4" s="9" t="s">
+        <v>520</v>
       </c>
       <c r="M4" s="3"/>
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
-      <c r="R4" s="9"/>
+      <c r="R4" s="9" t="s">
+        <v>628</v>
+      </c>
     </row>
     <row r="5" spans="1:18" ht="91.95" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -3259,16 +3328,18 @@
       <c r="C5" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="D5" s="8"/>
+      <c r="D5" s="8" t="s">
+        <v>488</v>
+      </c>
       <c r="E5" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G5" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A5="",COUNTIF($A$2:$A$14,A5)&lt;&gt;1,LEFT(A5,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D5="retain",E5="statistical_results")),H5&lt;&gt;"",NOT(EXACT(H5,"not_applicable"))),AND(NOT(AND(D5="retain",E5="statistical_results")),I5&lt;&gt;"",NOT(EXACT(I5,"not_applicable"))),AND(NOT(AND(D5="retain",E5="statistical_results")),J5&lt;&gt;"",NOT(EXACT(J5,"not_applicable"))),AND(NOT(AND(D5="retain",OR(E5="report_internal_inconsistency",E5="plan_material"))),K5&lt;&gt;"",NOT(EXACT(K5,"not_applicable"))),AND(NOT(AND(D5="retain",E5="protocol_report")),L5&lt;&gt;"",NOT(EXACT(L5,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D5,"retain"),EXACT(D5,"exclude"),EXACT(D5,"discuss"))),NOT(OR(EXACT(E5,"statistical_results"),EXACT(E5,"report_internal_inconsistency"),EXACT(E5,"plan_material"),EXACT(E5,"protocol_report"))),AND(AND(D5="retain",E5="statistical_results"),NOT(OR(EXACT(H5,"confirmed_issue"),EXACT(H5,"probable_issue"),EXACT(H5,"not_issue"),EXACT(H5,"indeterminate")))),AND(AND(D5="retain",E5="statistical_results"),NOT(OR(EXACT(I5,"substantive"),EXACT(I5,"minor_presentation"),EXACT(I5,"indeterminate")))),AND(AND(D5="retain",E5="statistical_results"),J5&lt;&gt;"",NOT(OR(EXACT(J5,"direct"),EXACT(J5,"possible"),EXACT(J5,"unlikely"),EXACT(J5,"unknown")))),AND(AND(D5="retain",OR(E5="report_internal_inconsistency",E5="plan_material")),NOT(OR(EXACT(K5,"substantive_inconsistency"),EXACT(K5,"minor_presentation"),EXACT(K5,"non_inconsistency"),EXACT(K5,"indeterminate")))),AND(AND(D5="retain",E5="protocol_report"),L5&lt;&gt;"",NOT(OR(EXACT(L5,"substantive_difference"),EXACT(L5,"minor_presentation"),EXACT(L5,"version_timing"),EXACT(L5,"non_inconsistency"),EXACT(L5,"indeterminate"))))),"CHECK FIELDS",IF(AND(F5&lt;&gt;"",NOT(OR(EXACT(F5,"no"),EXACT(F5,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F5,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H5" s="8" t="str">
         <f t="shared" si="0"/>
@@ -3287,15 +3358,17 @@
         <v>not_applicable</v>
       </c>
       <c r="L5" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+        <f t="shared" ref="L2:L14" si="4">IF(AND(OR(D5="retain",D5=""),E5="protocol_report"),"","not_applicable")</f>
+        <v>not_applicable</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
-      <c r="R5" s="9"/>
+      <c r="R5" s="9" t="s">
+        <v>630</v>
+      </c>
     </row>
     <row r="6" spans="1:18" ht="91.95" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -3307,16 +3380,18 @@
       <c r="C6" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D6" s="8"/>
+      <c r="D6" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E6" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G6" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A6="",COUNTIF($A$2:$A$14,A6)&lt;&gt;1,LEFT(A6,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D6="retain",E6="statistical_results")),H6&lt;&gt;"",NOT(EXACT(H6,"not_applicable"))),AND(NOT(AND(D6="retain",E6="statistical_results")),I6&lt;&gt;"",NOT(EXACT(I6,"not_applicable"))),AND(NOT(AND(D6="retain",E6="statistical_results")),J6&lt;&gt;"",NOT(EXACT(J6,"not_applicable"))),AND(NOT(AND(D6="retain",OR(E6="report_internal_inconsistency",E6="plan_material"))),K6&lt;&gt;"",NOT(EXACT(K6,"not_applicable"))),AND(NOT(AND(D6="retain",E6="protocol_report")),L6&lt;&gt;"",NOT(EXACT(L6,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D6,"retain"),EXACT(D6,"exclude"),EXACT(D6,"discuss"))),NOT(OR(EXACT(E6,"statistical_results"),EXACT(E6,"report_internal_inconsistency"),EXACT(E6,"plan_material"),EXACT(E6,"protocol_report"))),AND(AND(D6="retain",E6="statistical_results"),NOT(OR(EXACT(H6,"confirmed_issue"),EXACT(H6,"probable_issue"),EXACT(H6,"not_issue"),EXACT(H6,"indeterminate")))),AND(AND(D6="retain",E6="statistical_results"),NOT(OR(EXACT(I6,"substantive"),EXACT(I6,"minor_presentation"),EXACT(I6,"indeterminate")))),AND(AND(D6="retain",E6="statistical_results"),J6&lt;&gt;"",NOT(OR(EXACT(J6,"direct"),EXACT(J6,"possible"),EXACT(J6,"unlikely"),EXACT(J6,"unknown")))),AND(AND(D6="retain",OR(E6="report_internal_inconsistency",E6="plan_material")),NOT(OR(EXACT(K6,"substantive_inconsistency"),EXACT(K6,"minor_presentation"),EXACT(K6,"non_inconsistency"),EXACT(K6,"indeterminate")))),AND(AND(D6="retain",E6="protocol_report"),L6&lt;&gt;"",NOT(OR(EXACT(L6,"substantive_difference"),EXACT(L6,"minor_presentation"),EXACT(L6,"version_timing"),EXACT(L6,"non_inconsistency"),EXACT(L6,"indeterminate"))))),"CHECK FIELDS",IF(AND(F6&lt;&gt;"",NOT(OR(EXACT(F6,"no"),EXACT(F6,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F6,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H6" s="8" t="str">
         <f t="shared" si="0"/>
@@ -3334,16 +3409,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L6" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L6" s="9" t="s">
+        <v>526</v>
       </c>
       <c r="M6" s="3"/>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
-      <c r="R6" s="9"/>
+      <c r="R6" s="9" t="s">
+        <v>632</v>
+      </c>
     </row>
     <row r="7" spans="1:18" ht="91.95" customHeight="1">
       <c r="A7" s="1" t="s">
@@ -3355,16 +3431,18 @@
       <c r="C7" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="D7" s="8"/>
+      <c r="D7" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E7" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G7" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A7="",COUNTIF($A$2:$A$14,A7)&lt;&gt;1,LEFT(A7,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D7="retain",E7="statistical_results")),H7&lt;&gt;"",NOT(EXACT(H7,"not_applicable"))),AND(NOT(AND(D7="retain",E7="statistical_results")),I7&lt;&gt;"",NOT(EXACT(I7,"not_applicable"))),AND(NOT(AND(D7="retain",E7="statistical_results")),J7&lt;&gt;"",NOT(EXACT(J7,"not_applicable"))),AND(NOT(AND(D7="retain",OR(E7="report_internal_inconsistency",E7="plan_material"))),K7&lt;&gt;"",NOT(EXACT(K7,"not_applicable"))),AND(NOT(AND(D7="retain",E7="protocol_report")),L7&lt;&gt;"",NOT(EXACT(L7,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D7,"retain"),EXACT(D7,"exclude"),EXACT(D7,"discuss"))),NOT(OR(EXACT(E7,"statistical_results"),EXACT(E7,"report_internal_inconsistency"),EXACT(E7,"plan_material"),EXACT(E7,"protocol_report"))),AND(AND(D7="retain",E7="statistical_results"),NOT(OR(EXACT(H7,"confirmed_issue"),EXACT(H7,"probable_issue"),EXACT(H7,"not_issue"),EXACT(H7,"indeterminate")))),AND(AND(D7="retain",E7="statistical_results"),NOT(OR(EXACT(I7,"substantive"),EXACT(I7,"minor_presentation"),EXACT(I7,"indeterminate")))),AND(AND(D7="retain",E7="statistical_results"),J7&lt;&gt;"",NOT(OR(EXACT(J7,"direct"),EXACT(J7,"possible"),EXACT(J7,"unlikely"),EXACT(J7,"unknown")))),AND(AND(D7="retain",OR(E7="report_internal_inconsistency",E7="plan_material")),NOT(OR(EXACT(K7,"substantive_inconsistency"),EXACT(K7,"minor_presentation"),EXACT(K7,"non_inconsistency"),EXACT(K7,"indeterminate")))),AND(AND(D7="retain",E7="protocol_report"),L7&lt;&gt;"",NOT(OR(EXACT(L7,"substantive_difference"),EXACT(L7,"minor_presentation"),EXACT(L7,"version_timing"),EXACT(L7,"non_inconsistency"),EXACT(L7,"indeterminate"))))),"CHECK FIELDS",IF(AND(F7&lt;&gt;"",NOT(OR(EXACT(F7,"no"),EXACT(F7,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F7,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H7" s="8" t="str">
         <f t="shared" si="0"/>
@@ -3382,16 +3460,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L7" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L7" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M7" s="1"/>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
-      <c r="R7" s="9"/>
+      <c r="R7" s="9" t="s">
+        <v>634</v>
+      </c>
     </row>
     <row r="8" spans="1:18" ht="91.95" customHeight="1">
       <c r="A8" s="3" t="s">
@@ -3403,16 +3482,18 @@
       <c r="C8" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="D8" s="8"/>
+      <c r="D8" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E8" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G8" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A8="",COUNTIF($A$2:$A$14,A8)&lt;&gt;1,LEFT(A8,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D8="retain",E8="statistical_results")),H8&lt;&gt;"",NOT(EXACT(H8,"not_applicable"))),AND(NOT(AND(D8="retain",E8="statistical_results")),I8&lt;&gt;"",NOT(EXACT(I8,"not_applicable"))),AND(NOT(AND(D8="retain",E8="statistical_results")),J8&lt;&gt;"",NOT(EXACT(J8,"not_applicable"))),AND(NOT(AND(D8="retain",OR(E8="report_internal_inconsistency",E8="plan_material"))),K8&lt;&gt;"",NOT(EXACT(K8,"not_applicable"))),AND(NOT(AND(D8="retain",E8="protocol_report")),L8&lt;&gt;"",NOT(EXACT(L8,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D8,"retain"),EXACT(D8,"exclude"),EXACT(D8,"discuss"))),NOT(OR(EXACT(E8,"statistical_results"),EXACT(E8,"report_internal_inconsistency"),EXACT(E8,"plan_material"),EXACT(E8,"protocol_report"))),AND(AND(D8="retain",E8="statistical_results"),NOT(OR(EXACT(H8,"confirmed_issue"),EXACT(H8,"probable_issue"),EXACT(H8,"not_issue"),EXACT(H8,"indeterminate")))),AND(AND(D8="retain",E8="statistical_results"),NOT(OR(EXACT(I8,"substantive"),EXACT(I8,"minor_presentation"),EXACT(I8,"indeterminate")))),AND(AND(D8="retain",E8="statistical_results"),J8&lt;&gt;"",NOT(OR(EXACT(J8,"direct"),EXACT(J8,"possible"),EXACT(J8,"unlikely"),EXACT(J8,"unknown")))),AND(AND(D8="retain",OR(E8="report_internal_inconsistency",E8="plan_material")),NOT(OR(EXACT(K8,"substantive_inconsistency"),EXACT(K8,"minor_presentation"),EXACT(K8,"non_inconsistency"),EXACT(K8,"indeterminate")))),AND(AND(D8="retain",E8="protocol_report"),L8&lt;&gt;"",NOT(OR(EXACT(L8,"substantive_difference"),EXACT(L8,"minor_presentation"),EXACT(L8,"version_timing"),EXACT(L8,"non_inconsistency"),EXACT(L8,"indeterminate"))))),"CHECK FIELDS",IF(AND(F8&lt;&gt;"",NOT(OR(EXACT(F8,"no"),EXACT(F8,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F8,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H8" s="8" t="str">
         <f t="shared" si="0"/>
@@ -3430,16 +3511,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L8" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L8" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M8" s="3"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
-      <c r="R8" s="9"/>
+      <c r="R8" s="9" t="s">
+        <v>636</v>
+      </c>
     </row>
     <row r="9" spans="1:18" ht="91.95" customHeight="1">
       <c r="A9" s="1" t="s">
@@ -3451,16 +3533,18 @@
       <c r="C9" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="D9" s="8"/>
+      <c r="D9" s="8" t="s">
+        <v>488</v>
+      </c>
       <c r="E9" s="8" t="s">
         <v>81</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G9" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A9="",COUNTIF($A$2:$A$14,A9)&lt;&gt;1,LEFT(A9,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D9="retain",E9="statistical_results")),H9&lt;&gt;"",NOT(EXACT(H9,"not_applicable"))),AND(NOT(AND(D9="retain",E9="statistical_results")),I9&lt;&gt;"",NOT(EXACT(I9,"not_applicable"))),AND(NOT(AND(D9="retain",E9="statistical_results")),J9&lt;&gt;"",NOT(EXACT(J9,"not_applicable"))),AND(NOT(AND(D9="retain",OR(E9="report_internal_inconsistency",E9="plan_material"))),K9&lt;&gt;"",NOT(EXACT(K9,"not_applicable"))),AND(NOT(AND(D9="retain",E9="protocol_report")),L9&lt;&gt;"",NOT(EXACT(L9,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D9,"retain"),EXACT(D9,"exclude"),EXACT(D9,"discuss"))),NOT(OR(EXACT(E9,"statistical_results"),EXACT(E9,"report_internal_inconsistency"),EXACT(E9,"plan_material"),EXACT(E9,"protocol_report"))),AND(AND(D9="retain",E9="statistical_results"),NOT(OR(EXACT(H9,"confirmed_issue"),EXACT(H9,"probable_issue"),EXACT(H9,"not_issue"),EXACT(H9,"indeterminate")))),AND(AND(D9="retain",E9="statistical_results"),NOT(OR(EXACT(I9,"substantive"),EXACT(I9,"minor_presentation"),EXACT(I9,"indeterminate")))),AND(AND(D9="retain",E9="statistical_results"),J9&lt;&gt;"",NOT(OR(EXACT(J9,"direct"),EXACT(J9,"possible"),EXACT(J9,"unlikely"),EXACT(J9,"unknown")))),AND(AND(D9="retain",OR(E9="report_internal_inconsistency",E9="plan_material")),NOT(OR(EXACT(K9,"substantive_inconsistency"),EXACT(K9,"minor_presentation"),EXACT(K9,"non_inconsistency"),EXACT(K9,"indeterminate")))),AND(AND(D9="retain",E9="protocol_report"),L9&lt;&gt;"",NOT(OR(EXACT(L9,"substantive_difference"),EXACT(L9,"minor_presentation"),EXACT(L9,"version_timing"),EXACT(L9,"non_inconsistency"),EXACT(L9,"indeterminate"))))),"CHECK FIELDS",IF(AND(F9&lt;&gt;"",NOT(OR(EXACT(F9,"no"),EXACT(F9,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F9,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H9" s="8" t="str">
         <f t="shared" si="0"/>
@@ -3476,7 +3560,7 @@
       </c>
       <c r="K9" s="8" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>not_applicable</v>
       </c>
       <c r="L9" s="9" t="str">
         <f t="shared" si="4"/>
@@ -3487,7 +3571,9 @@
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
-      <c r="R9" s="9"/>
+      <c r="R9" s="9" t="s">
+        <v>635</v>
+      </c>
     </row>
     <row r="10" spans="1:18" ht="91.95" customHeight="1">
       <c r="A10" s="3" t="s">
@@ -3499,28 +3585,27 @@
       <c r="C10" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="D10" s="8"/>
+      <c r="D10" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E10" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G10" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A10="",COUNTIF($A$2:$A$14,A10)&lt;&gt;1,LEFT(A10,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D10="retain",E10="statistical_results")),H10&lt;&gt;"",NOT(EXACT(H10,"not_applicable"))),AND(NOT(AND(D10="retain",E10="statistical_results")),I10&lt;&gt;"",NOT(EXACT(I10,"not_applicable"))),AND(NOT(AND(D10="retain",E10="statistical_results")),J10&lt;&gt;"",NOT(EXACT(J10,"not_applicable"))),AND(NOT(AND(D10="retain",OR(E10="report_internal_inconsistency",E10="plan_material"))),K10&lt;&gt;"",NOT(EXACT(K10,"not_applicable"))),AND(NOT(AND(D10="retain",E10="protocol_report")),L10&lt;&gt;"",NOT(EXACT(L10,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D10,"retain"),EXACT(D10,"exclude"),EXACT(D10,"discuss"))),NOT(OR(EXACT(E10,"statistical_results"),EXACT(E10,"report_internal_inconsistency"),EXACT(E10,"plan_material"),EXACT(E10,"protocol_report"))),AND(AND(D10="retain",E10="statistical_results"),NOT(OR(EXACT(H10,"confirmed_issue"),EXACT(H10,"probable_issue"),EXACT(H10,"not_issue"),EXACT(H10,"indeterminate")))),AND(AND(D10="retain",E10="statistical_results"),NOT(OR(EXACT(I10,"substantive"),EXACT(I10,"minor_presentation"),EXACT(I10,"indeterminate")))),AND(AND(D10="retain",E10="statistical_results"),J10&lt;&gt;"",NOT(OR(EXACT(J10,"direct"),EXACT(J10,"possible"),EXACT(J10,"unlikely"),EXACT(J10,"unknown")))),AND(AND(D10="retain",OR(E10="report_internal_inconsistency",E10="plan_material")),NOT(OR(EXACT(K10,"substantive_inconsistency"),EXACT(K10,"minor_presentation"),EXACT(K10,"non_inconsistency"),EXACT(K10,"indeterminate")))),AND(AND(D10="retain",E10="protocol_report"),L10&lt;&gt;"",NOT(OR(EXACT(L10,"substantive_difference"),EXACT(L10,"minor_presentation"),EXACT(L10,"version_timing"),EXACT(L10,"non_inconsistency"),EXACT(L10,"indeterminate"))))),"CHECK FIELDS",IF(AND(F10&lt;&gt;"",NOT(OR(EXACT(F10,"no"),EXACT(F10,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F10,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
-      </c>
-      <c r="H10" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I10" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J10" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+        <v>PRIMARY READY</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>518</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>534</v>
       </c>
       <c r="K10" s="8" t="str">
         <f t="shared" si="3"/>
@@ -3535,7 +3620,9 @@
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
-      <c r="R10" s="9"/>
+      <c r="R10" s="9" t="s">
+        <v>633</v>
+      </c>
     </row>
     <row r="11" spans="1:18" ht="91.95" customHeight="1">
       <c r="A11" s="1" t="s">
@@ -3547,28 +3634,30 @@
       <c r="C11" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="D11" s="8"/>
+      <c r="D11" s="8" t="s">
+        <v>488</v>
+      </c>
       <c r="E11" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G11" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A11="",COUNTIF($A$2:$A$14,A11)&lt;&gt;1,LEFT(A11,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D11="retain",E11="statistical_results")),H11&lt;&gt;"",NOT(EXACT(H11,"not_applicable"))),AND(NOT(AND(D11="retain",E11="statistical_results")),I11&lt;&gt;"",NOT(EXACT(I11,"not_applicable"))),AND(NOT(AND(D11="retain",E11="statistical_results")),J11&lt;&gt;"",NOT(EXACT(J11,"not_applicable"))),AND(NOT(AND(D11="retain",OR(E11="report_internal_inconsistency",E11="plan_material"))),K11&lt;&gt;"",NOT(EXACT(K11,"not_applicable"))),AND(NOT(AND(D11="retain",E11="protocol_report")),L11&lt;&gt;"",NOT(EXACT(L11,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D11,"retain"),EXACT(D11,"exclude"),EXACT(D11,"discuss"))),NOT(OR(EXACT(E11,"statistical_results"),EXACT(E11,"report_internal_inconsistency"),EXACT(E11,"plan_material"),EXACT(E11,"protocol_report"))),AND(AND(D11="retain",E11="statistical_results"),NOT(OR(EXACT(H11,"confirmed_issue"),EXACT(H11,"probable_issue"),EXACT(H11,"not_issue"),EXACT(H11,"indeterminate")))),AND(AND(D11="retain",E11="statistical_results"),NOT(OR(EXACT(I11,"substantive"),EXACT(I11,"minor_presentation"),EXACT(I11,"indeterminate")))),AND(AND(D11="retain",E11="statistical_results"),J11&lt;&gt;"",NOT(OR(EXACT(J11,"direct"),EXACT(J11,"possible"),EXACT(J11,"unlikely"),EXACT(J11,"unknown")))),AND(AND(D11="retain",OR(E11="report_internal_inconsistency",E11="plan_material")),NOT(OR(EXACT(K11,"substantive_inconsistency"),EXACT(K11,"minor_presentation"),EXACT(K11,"non_inconsistency"),EXACT(K11,"indeterminate")))),AND(AND(D11="retain",E11="protocol_report"),L11&lt;&gt;"",NOT(OR(EXACT(L11,"substantive_difference"),EXACT(L11,"minor_presentation"),EXACT(L11,"version_timing"),EXACT(L11,"non_inconsistency"),EXACT(L11,"indeterminate"))))),"CHECK FIELDS",IF(AND(F11&lt;&gt;"",NOT(OR(EXACT(F11,"no"),EXACT(F11,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F11,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H11" s="8" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>not_applicable</v>
       </c>
       <c r="I11" s="8" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>not_applicable</v>
       </c>
       <c r="J11" s="9" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>not_applicable</v>
       </c>
       <c r="K11" s="8" t="str">
         <f t="shared" si="3"/>
@@ -3583,7 +3672,9 @@
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
-      <c r="R11" s="9"/>
+      <c r="R11" s="9" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="12" spans="1:18" ht="91.95" customHeight="1">
       <c r="A12" s="3" t="s">
@@ -3595,28 +3686,27 @@
       <c r="C12" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="D12" s="8"/>
+      <c r="D12" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E12" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G12" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A12="",COUNTIF($A$2:$A$14,A12)&lt;&gt;1,LEFT(A12,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D12="retain",E12="statistical_results")),H12&lt;&gt;"",NOT(EXACT(H12,"not_applicable"))),AND(NOT(AND(D12="retain",E12="statistical_results")),I12&lt;&gt;"",NOT(EXACT(I12,"not_applicable"))),AND(NOT(AND(D12="retain",E12="statistical_results")),J12&lt;&gt;"",NOT(EXACT(J12,"not_applicable"))),AND(NOT(AND(D12="retain",OR(E12="report_internal_inconsistency",E12="plan_material"))),K12&lt;&gt;"",NOT(EXACT(K12,"not_applicable"))),AND(NOT(AND(D12="retain",E12="protocol_report")),L12&lt;&gt;"",NOT(EXACT(L12,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D12,"retain"),EXACT(D12,"exclude"),EXACT(D12,"discuss"))),NOT(OR(EXACT(E12,"statistical_results"),EXACT(E12,"report_internal_inconsistency"),EXACT(E12,"plan_material"),EXACT(E12,"protocol_report"))),AND(AND(D12="retain",E12="statistical_results"),NOT(OR(EXACT(H12,"confirmed_issue"),EXACT(H12,"probable_issue"),EXACT(H12,"not_issue"),EXACT(H12,"indeterminate")))),AND(AND(D12="retain",E12="statistical_results"),NOT(OR(EXACT(I12,"substantive"),EXACT(I12,"minor_presentation"),EXACT(I12,"indeterminate")))),AND(AND(D12="retain",E12="statistical_results"),J12&lt;&gt;"",NOT(OR(EXACT(J12,"direct"),EXACT(J12,"possible"),EXACT(J12,"unlikely"),EXACT(J12,"unknown")))),AND(AND(D12="retain",OR(E12="report_internal_inconsistency",E12="plan_material")),NOT(OR(EXACT(K12,"substantive_inconsistency"),EXACT(K12,"minor_presentation"),EXACT(K12,"non_inconsistency"),EXACT(K12,"indeterminate")))),AND(AND(D12="retain",E12="protocol_report"),L12&lt;&gt;"",NOT(OR(EXACT(L12,"substantive_difference"),EXACT(L12,"minor_presentation"),EXACT(L12,"version_timing"),EXACT(L12,"non_inconsistency"),EXACT(L12,"indeterminate"))))),"CHECK FIELDS",IF(AND(F12&lt;&gt;"",NOT(OR(EXACT(F12,"no"),EXACT(F12,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F12,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
-      </c>
-      <c r="H12" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I12" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J12" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+        <v>PRIMARY READY</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>536</v>
       </c>
       <c r="K12" s="8" t="str">
         <f t="shared" si="3"/>
@@ -3631,7 +3721,9 @@
       <c r="O12" s="4"/>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
-      <c r="R12" s="9"/>
+      <c r="R12" s="9" t="s">
+        <v>629</v>
+      </c>
     </row>
     <row r="13" spans="1:18" ht="91.95" customHeight="1">
       <c r="A13" s="1" t="s">
@@ -3643,28 +3735,27 @@
       <c r="C13" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="D13" s="8"/>
+      <c r="D13" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E13" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G13" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A13="",COUNTIF($A$2:$A$14,A13)&lt;&gt;1,LEFT(A13,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D13="retain",E13="statistical_results")),H13&lt;&gt;"",NOT(EXACT(H13,"not_applicable"))),AND(NOT(AND(D13="retain",E13="statistical_results")),I13&lt;&gt;"",NOT(EXACT(I13,"not_applicable"))),AND(NOT(AND(D13="retain",E13="statistical_results")),J13&lt;&gt;"",NOT(EXACT(J13,"not_applicable"))),AND(NOT(AND(D13="retain",OR(E13="report_internal_inconsistency",E13="plan_material"))),K13&lt;&gt;"",NOT(EXACT(K13,"not_applicable"))),AND(NOT(AND(D13="retain",E13="protocol_report")),L13&lt;&gt;"",NOT(EXACT(L13,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D13,"retain"),EXACT(D13,"exclude"),EXACT(D13,"discuss"))),NOT(OR(EXACT(E13,"statistical_results"),EXACT(E13,"report_internal_inconsistency"),EXACT(E13,"plan_material"),EXACT(E13,"protocol_report"))),AND(AND(D13="retain",E13="statistical_results"),NOT(OR(EXACT(H13,"confirmed_issue"),EXACT(H13,"probable_issue"),EXACT(H13,"not_issue"),EXACT(H13,"indeterminate")))),AND(AND(D13="retain",E13="statistical_results"),NOT(OR(EXACT(I13,"substantive"),EXACT(I13,"minor_presentation"),EXACT(I13,"indeterminate")))),AND(AND(D13="retain",E13="statistical_results"),J13&lt;&gt;"",NOT(OR(EXACT(J13,"direct"),EXACT(J13,"possible"),EXACT(J13,"unlikely"),EXACT(J13,"unknown")))),AND(AND(D13="retain",OR(E13="report_internal_inconsistency",E13="plan_material")),NOT(OR(EXACT(K13,"substantive_inconsistency"),EXACT(K13,"minor_presentation"),EXACT(K13,"non_inconsistency"),EXACT(K13,"indeterminate")))),AND(AND(D13="retain",E13="protocol_report"),L13&lt;&gt;"",NOT(OR(EXACT(L13,"substantive_difference"),EXACT(L13,"minor_presentation"),EXACT(L13,"version_timing"),EXACT(L13,"non_inconsistency"),EXACT(L13,"indeterminate"))))),"CHECK FIELDS",IF(AND(F13&lt;&gt;"",NOT(OR(EXACT(F13,"no"),EXACT(F13,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F13,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
-      </c>
-      <c r="H13" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I13" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J13" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+        <v>PRIMARY READY</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>524</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>534</v>
       </c>
       <c r="K13" s="8" t="str">
         <f t="shared" si="3"/>
@@ -3679,7 +3770,9 @@
       <c r="O13" s="4"/>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
-      <c r="R13" s="9"/>
+      <c r="R13" s="9" t="s">
+        <v>627</v>
+      </c>
     </row>
     <row r="14" spans="1:18" ht="91.95" customHeight="1">
       <c r="A14" s="3" t="s">
@@ -3691,28 +3784,27 @@
       <c r="C14" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="D14" s="8"/>
+      <c r="D14" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E14" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G14" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A14="",COUNTIF($A$2:$A$14,A14)&lt;&gt;1,LEFT(A14,LEN("2025::jama.2025.19563::"))&lt;&gt;"2025::jama.2025.19563::"),"CHECK KEY",IF(OR(AND(NOT(AND(D14="retain",E14="statistical_results")),H14&lt;&gt;"",NOT(EXACT(H14,"not_applicable"))),AND(NOT(AND(D14="retain",E14="statistical_results")),I14&lt;&gt;"",NOT(EXACT(I14,"not_applicable"))),AND(NOT(AND(D14="retain",E14="statistical_results")),J14&lt;&gt;"",NOT(EXACT(J14,"not_applicable"))),AND(NOT(AND(D14="retain",OR(E14="report_internal_inconsistency",E14="plan_material"))),K14&lt;&gt;"",NOT(EXACT(K14,"not_applicable"))),AND(NOT(AND(D14="retain",E14="protocol_report")),L14&lt;&gt;"",NOT(EXACT(L14,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D14,"retain"),EXACT(D14,"exclude"),EXACT(D14,"discuss"))),NOT(OR(EXACT(E14,"statistical_results"),EXACT(E14,"report_internal_inconsistency"),EXACT(E14,"plan_material"),EXACT(E14,"protocol_report"))),AND(AND(D14="retain",E14="statistical_results"),NOT(OR(EXACT(H14,"confirmed_issue"),EXACT(H14,"probable_issue"),EXACT(H14,"not_issue"),EXACT(H14,"indeterminate")))),AND(AND(D14="retain",E14="statistical_results"),NOT(OR(EXACT(I14,"substantive"),EXACT(I14,"minor_presentation"),EXACT(I14,"indeterminate")))),AND(AND(D14="retain",E14="statistical_results"),J14&lt;&gt;"",NOT(OR(EXACT(J14,"direct"),EXACT(J14,"possible"),EXACT(J14,"unlikely"),EXACT(J14,"unknown")))),AND(AND(D14="retain",OR(E14="report_internal_inconsistency",E14="plan_material")),NOT(OR(EXACT(K14,"substantive_inconsistency"),EXACT(K14,"minor_presentation"),EXACT(K14,"non_inconsistency"),EXACT(K14,"indeterminate")))),AND(AND(D14="retain",E14="protocol_report"),L14&lt;&gt;"",NOT(OR(EXACT(L14,"substantive_difference"),EXACT(L14,"minor_presentation"),EXACT(L14,"version_timing"),EXACT(L14,"non_inconsistency"),EXACT(L14,"indeterminate"))))),"CHECK FIELDS",IF(AND(F14&lt;&gt;"",NOT(OR(EXACT(F14,"no"),EXACT(F14,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F14,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
-      </c>
-      <c r="H14" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I14" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J14" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+        <v>PRIMARY READY</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>524</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>534</v>
       </c>
       <c r="K14" s="8" t="str">
         <f t="shared" si="3"/>
@@ -3727,7 +3819,9 @@
       <c r="O14" s="4"/>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
-      <c r="R14" s="9"/>
+      <c r="R14" s="9" t="s">
+        <v>625</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:R14" xr:uid="{00000000-0009-0000-0000-000009000000}"/>
@@ -3858,35 +3952,34 @@
       <c r="C2" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="D2" s="8"/>
+      <c r="D2" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E2" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G2" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A2="",COUNTIF($A$2:$A$8,A2)&lt;&gt;1,LEFT(A2,LEN("2025::jama.2025.19843::"))&lt;&gt;"2025::jama.2025.19843::"),"CHECK KEY",IF(OR(AND(NOT(AND(D2="retain",E2="statistical_results")),H2&lt;&gt;"",NOT(EXACT(H2,"not_applicable"))),AND(NOT(AND(D2="retain",E2="statistical_results")),I2&lt;&gt;"",NOT(EXACT(I2,"not_applicable"))),AND(NOT(AND(D2="retain",E2="statistical_results")),J2&lt;&gt;"",NOT(EXACT(J2,"not_applicable"))),AND(NOT(AND(D2="retain",OR(E2="report_internal_inconsistency",E2="plan_material"))),K2&lt;&gt;"",NOT(EXACT(K2,"not_applicable"))),AND(NOT(AND(D2="retain",E2="protocol_report")),L2&lt;&gt;"",NOT(EXACT(L2,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D2,"retain"),EXACT(D2,"exclude"),EXACT(D2,"discuss"))),NOT(OR(EXACT(E2,"statistical_results"),EXACT(E2,"report_internal_inconsistency"),EXACT(E2,"plan_material"),EXACT(E2,"protocol_report"))),AND(AND(D2="retain",E2="statistical_results"),NOT(OR(EXACT(H2,"confirmed_issue"),EXACT(H2,"probable_issue"),EXACT(H2,"not_issue"),EXACT(H2,"indeterminate")))),AND(AND(D2="retain",E2="statistical_results"),NOT(OR(EXACT(I2,"substantive"),EXACT(I2,"minor_presentation"),EXACT(I2,"indeterminate")))),AND(AND(D2="retain",E2="statistical_results"),J2&lt;&gt;"",NOT(OR(EXACT(J2,"direct"),EXACT(J2,"possible"),EXACT(J2,"unlikely"),EXACT(J2,"unknown")))),AND(AND(D2="retain",OR(E2="report_internal_inconsistency",E2="plan_material")),NOT(OR(EXACT(K2,"substantive_inconsistency"),EXACT(K2,"minor_presentation"),EXACT(K2,"non_inconsistency"),EXACT(K2,"indeterminate")))),AND(AND(D2="retain",E2="protocol_report"),L2&lt;&gt;"",NOT(OR(EXACT(L2,"substantive_difference"),EXACT(L2,"minor_presentation"),EXACT(L2,"version_timing"),EXACT(L2,"non_inconsistency"),EXACT(L2,"indeterminate"))))),"CHECK FIELDS",IF(AND(F2&lt;&gt;"",NOT(OR(EXACT(F2,"no"),EXACT(F2,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F2,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
-      </c>
-      <c r="H2" s="8" t="str">
-        <f t="shared" ref="H2:H8" si="0">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
-        <v/>
-      </c>
-      <c r="I2" s="8" t="str">
-        <f t="shared" ref="I2:I8" si="1">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
-        <v/>
-      </c>
-      <c r="J2" s="9" t="str">
-        <f t="shared" ref="J2:J8" si="2">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
-        <v/>
+        <v>PRIMARY READY</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>524</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>534</v>
       </c>
       <c r="K2" s="8" t="str">
-        <f t="shared" ref="K2:K8" si="3">IF(AND(OR(D2="retain",D2=""),OR(E2="report_internal_inconsistency",E2="plan_material")),"","not_applicable")</f>
+        <f t="shared" ref="K2:K8" si="0">IF(AND(OR(D2="retain",D2=""),OR(E2="report_internal_inconsistency",E2="plan_material")),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="L2" s="9" t="str">
-        <f t="shared" ref="L2:L8" si="4">IF(AND(OR(D2="retain",D2=""),E2="protocol_report"),"","not_applicable")</f>
+        <f t="shared" ref="L2:L8" si="1">IF(AND(OR(D2="retain",D2=""),E2="protocol_report"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="M2" s="3"/>
@@ -3894,7 +3987,9 @@
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
-      <c r="R2" s="9"/>
+      <c r="R2" s="9" t="s">
+        <v>637</v>
+      </c>
     </row>
     <row r="3" spans="1:18" ht="91.95" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -3906,43 +4001,46 @@
       <c r="C3" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="D3" s="8"/>
+      <c r="D3" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E3" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G3" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A3="",COUNTIF($A$2:$A$8,A3)&lt;&gt;1,LEFT(A3,LEN("2025::jama.2025.19843::"))&lt;&gt;"2025::jama.2025.19843::"),"CHECK KEY",IF(OR(AND(NOT(AND(D3="retain",E3="statistical_results")),H3&lt;&gt;"",NOT(EXACT(H3,"not_applicable"))),AND(NOT(AND(D3="retain",E3="statistical_results")),I3&lt;&gt;"",NOT(EXACT(I3,"not_applicable"))),AND(NOT(AND(D3="retain",E3="statistical_results")),J3&lt;&gt;"",NOT(EXACT(J3,"not_applicable"))),AND(NOT(AND(D3="retain",OR(E3="report_internal_inconsistency",E3="plan_material"))),K3&lt;&gt;"",NOT(EXACT(K3,"not_applicable"))),AND(NOT(AND(D3="retain",E3="protocol_report")),L3&lt;&gt;"",NOT(EXACT(L3,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D3,"retain"),EXACT(D3,"exclude"),EXACT(D3,"discuss"))),NOT(OR(EXACT(E3,"statistical_results"),EXACT(E3,"report_internal_inconsistency"),EXACT(E3,"plan_material"),EXACT(E3,"protocol_report"))),AND(AND(D3="retain",E3="statistical_results"),NOT(OR(EXACT(H3,"confirmed_issue"),EXACT(H3,"probable_issue"),EXACT(H3,"not_issue"),EXACT(H3,"indeterminate")))),AND(AND(D3="retain",E3="statistical_results"),NOT(OR(EXACT(I3,"substantive"),EXACT(I3,"minor_presentation"),EXACT(I3,"indeterminate")))),AND(AND(D3="retain",E3="statistical_results"),J3&lt;&gt;"",NOT(OR(EXACT(J3,"direct"),EXACT(J3,"possible"),EXACT(J3,"unlikely"),EXACT(J3,"unknown")))),AND(AND(D3="retain",OR(E3="report_internal_inconsistency",E3="plan_material")),NOT(OR(EXACT(K3,"substantive_inconsistency"),EXACT(K3,"minor_presentation"),EXACT(K3,"non_inconsistency"),EXACT(K3,"indeterminate")))),AND(AND(D3="retain",E3="protocol_report"),L3&lt;&gt;"",NOT(OR(EXACT(L3,"substantive_difference"),EXACT(L3,"minor_presentation"),EXACT(L3,"version_timing"),EXACT(L3,"non_inconsistency"),EXACT(L3,"indeterminate"))))),"CHECK FIELDS",IF(AND(F3&lt;&gt;"",NOT(OR(EXACT(F3,"no"),EXACT(F3,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F3,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H3" s="8" t="str">
+        <f t="shared" ref="H2:H8" si="2">IF(AND(OR(D3="retain",D3=""),E3="statistical_results"),"","not_applicable")</f>
+        <v>not_applicable</v>
+      </c>
+      <c r="I3" s="8" t="str">
+        <f t="shared" ref="I2:I8" si="3">IF(AND(OR(D3="retain",D3=""),E3="statistical_results"),"","not_applicable")</f>
+        <v>not_applicable</v>
+      </c>
+      <c r="J3" s="9" t="str">
+        <f t="shared" ref="J2:J8" si="4">IF(AND(OR(D3="retain",D3=""),E3="statistical_results"),"","not_applicable")</f>
+        <v>not_applicable</v>
+      </c>
+      <c r="K3" s="8" t="str">
         <f t="shared" si="0"/>
         <v>not_applicable</v>
       </c>
-      <c r="I3" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="J3" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="K3" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="L3" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L3" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M3" s="1"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="9"/>
+      <c r="R3" s="9" t="s">
+        <v>639</v>
+      </c>
     </row>
     <row r="4" spans="1:18" ht="91.95" customHeight="1">
       <c r="A4" s="3" t="s">
@@ -3954,43 +4052,46 @@
       <c r="C4" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="D4" s="8"/>
+      <c r="D4" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E4" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G4" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A4="",COUNTIF($A$2:$A$8,A4)&lt;&gt;1,LEFT(A4,LEN("2025::jama.2025.19843::"))&lt;&gt;"2025::jama.2025.19843::"),"CHECK KEY",IF(OR(AND(NOT(AND(D4="retain",E4="statistical_results")),H4&lt;&gt;"",NOT(EXACT(H4,"not_applicable"))),AND(NOT(AND(D4="retain",E4="statistical_results")),I4&lt;&gt;"",NOT(EXACT(I4,"not_applicable"))),AND(NOT(AND(D4="retain",E4="statistical_results")),J4&lt;&gt;"",NOT(EXACT(J4,"not_applicable"))),AND(NOT(AND(D4="retain",OR(E4="report_internal_inconsistency",E4="plan_material"))),K4&lt;&gt;"",NOT(EXACT(K4,"not_applicable"))),AND(NOT(AND(D4="retain",E4="protocol_report")),L4&lt;&gt;"",NOT(EXACT(L4,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D4,"retain"),EXACT(D4,"exclude"),EXACT(D4,"discuss"))),NOT(OR(EXACT(E4,"statistical_results"),EXACT(E4,"report_internal_inconsistency"),EXACT(E4,"plan_material"),EXACT(E4,"protocol_report"))),AND(AND(D4="retain",E4="statistical_results"),NOT(OR(EXACT(H4,"confirmed_issue"),EXACT(H4,"probable_issue"),EXACT(H4,"not_issue"),EXACT(H4,"indeterminate")))),AND(AND(D4="retain",E4="statistical_results"),NOT(OR(EXACT(I4,"substantive"),EXACT(I4,"minor_presentation"),EXACT(I4,"indeterminate")))),AND(AND(D4="retain",E4="statistical_results"),J4&lt;&gt;"",NOT(OR(EXACT(J4,"direct"),EXACT(J4,"possible"),EXACT(J4,"unlikely"),EXACT(J4,"unknown")))),AND(AND(D4="retain",OR(E4="report_internal_inconsistency",E4="plan_material")),NOT(OR(EXACT(K4,"substantive_inconsistency"),EXACT(K4,"minor_presentation"),EXACT(K4,"non_inconsistency"),EXACT(K4,"indeterminate")))),AND(AND(D4="retain",E4="protocol_report"),L4&lt;&gt;"",NOT(OR(EXACT(L4,"substantive_difference"),EXACT(L4,"minor_presentation"),EXACT(L4,"version_timing"),EXACT(L4,"non_inconsistency"),EXACT(L4,"indeterminate"))))),"CHECK FIELDS",IF(AND(F4&lt;&gt;"",NOT(OR(EXACT(F4,"no"),EXACT(F4,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F4,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H4" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="I4" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="J4" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="K4" s="8" t="str">
         <f t="shared" si="0"/>
         <v>not_applicable</v>
       </c>
-      <c r="I4" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="J4" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="K4" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="L4" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L4" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M4" s="3"/>
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
-      <c r="R4" s="9"/>
+      <c r="R4" s="9" t="s">
+        <v>641</v>
+      </c>
     </row>
     <row r="5" spans="1:18" ht="91.95" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -4002,43 +4103,45 @@
       <c r="C5" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="D5" s="8"/>
+      <c r="D5" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E5" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G5" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A5="",COUNTIF($A$2:$A$8,A5)&lt;&gt;1,LEFT(A5,LEN("2025::jama.2025.19843::"))&lt;&gt;"2025::jama.2025.19843::"),"CHECK KEY",IF(OR(AND(NOT(AND(D5="retain",E5="statistical_results")),H5&lt;&gt;"",NOT(EXACT(H5,"not_applicable"))),AND(NOT(AND(D5="retain",E5="statistical_results")),I5&lt;&gt;"",NOT(EXACT(I5,"not_applicable"))),AND(NOT(AND(D5="retain",E5="statistical_results")),J5&lt;&gt;"",NOT(EXACT(J5,"not_applicable"))),AND(NOT(AND(D5="retain",OR(E5="report_internal_inconsistency",E5="plan_material"))),K5&lt;&gt;"",NOT(EXACT(K5,"not_applicable"))),AND(NOT(AND(D5="retain",E5="protocol_report")),L5&lt;&gt;"",NOT(EXACT(L5,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D5,"retain"),EXACT(D5,"exclude"),EXACT(D5,"discuss"))),NOT(OR(EXACT(E5,"statistical_results"),EXACT(E5,"report_internal_inconsistency"),EXACT(E5,"plan_material"),EXACT(E5,"protocol_report"))),AND(AND(D5="retain",E5="statistical_results"),NOT(OR(EXACT(H5,"confirmed_issue"),EXACT(H5,"probable_issue"),EXACT(H5,"not_issue"),EXACT(H5,"indeterminate")))),AND(AND(D5="retain",E5="statistical_results"),NOT(OR(EXACT(I5,"substantive"),EXACT(I5,"minor_presentation"),EXACT(I5,"indeterminate")))),AND(AND(D5="retain",E5="statistical_results"),J5&lt;&gt;"",NOT(OR(EXACT(J5,"direct"),EXACT(J5,"possible"),EXACT(J5,"unlikely"),EXACT(J5,"unknown")))),AND(AND(D5="retain",OR(E5="report_internal_inconsistency",E5="plan_material")),NOT(OR(EXACT(K5,"substantive_inconsistency"),EXACT(K5,"minor_presentation"),EXACT(K5,"non_inconsistency"),EXACT(K5,"indeterminate")))),AND(AND(D5="retain",E5="protocol_report"),L5&lt;&gt;"",NOT(OR(EXACT(L5,"substantive_difference"),EXACT(L5,"minor_presentation"),EXACT(L5,"version_timing"),EXACT(L5,"non_inconsistency"),EXACT(L5,"indeterminate"))))),"CHECK FIELDS",IF(AND(F5&lt;&gt;"",NOT(OR(EXACT(F5,"no"),EXACT(F5,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F5,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
-      </c>
-      <c r="H5" s="8" t="str">
+        <v>PRIMARY READY</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>520</v>
+      </c>
+      <c r="I5" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="J5" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="K5" s="8" t="str">
         <f t="shared" si="0"/>
         <v>not_applicable</v>
       </c>
-      <c r="I5" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="J5" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="K5" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="L5" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L5" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
-      <c r="R5" s="9"/>
+      <c r="R5" s="9" t="s">
+        <v>643</v>
+      </c>
     </row>
     <row r="6" spans="1:18" ht="91.95" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -4050,43 +4153,46 @@
       <c r="C6" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="D6" s="8"/>
+      <c r="D6" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E6" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G6" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A6="",COUNTIF($A$2:$A$8,A6)&lt;&gt;1,LEFT(A6,LEN("2025::jama.2025.19843::"))&lt;&gt;"2025::jama.2025.19843::"),"CHECK KEY",IF(OR(AND(NOT(AND(D6="retain",E6="statistical_results")),H6&lt;&gt;"",NOT(EXACT(H6,"not_applicable"))),AND(NOT(AND(D6="retain",E6="statistical_results")),I6&lt;&gt;"",NOT(EXACT(I6,"not_applicable"))),AND(NOT(AND(D6="retain",E6="statistical_results")),J6&lt;&gt;"",NOT(EXACT(J6,"not_applicable"))),AND(NOT(AND(D6="retain",OR(E6="report_internal_inconsistency",E6="plan_material"))),K6&lt;&gt;"",NOT(EXACT(K6,"not_applicable"))),AND(NOT(AND(D6="retain",E6="protocol_report")),L6&lt;&gt;"",NOT(EXACT(L6,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D6,"retain"),EXACT(D6,"exclude"),EXACT(D6,"discuss"))),NOT(OR(EXACT(E6,"statistical_results"),EXACT(E6,"report_internal_inconsistency"),EXACT(E6,"plan_material"),EXACT(E6,"protocol_report"))),AND(AND(D6="retain",E6="statistical_results"),NOT(OR(EXACT(H6,"confirmed_issue"),EXACT(H6,"probable_issue"),EXACT(H6,"not_issue"),EXACT(H6,"indeterminate")))),AND(AND(D6="retain",E6="statistical_results"),NOT(OR(EXACT(I6,"substantive"),EXACT(I6,"minor_presentation"),EXACT(I6,"indeterminate")))),AND(AND(D6="retain",E6="statistical_results"),J6&lt;&gt;"",NOT(OR(EXACT(J6,"direct"),EXACT(J6,"possible"),EXACT(J6,"unlikely"),EXACT(J6,"unknown")))),AND(AND(D6="retain",OR(E6="report_internal_inconsistency",E6="plan_material")),NOT(OR(EXACT(K6,"substantive_inconsistency"),EXACT(K6,"minor_presentation"),EXACT(K6,"non_inconsistency"),EXACT(K6,"indeterminate")))),AND(AND(D6="retain",E6="protocol_report"),L6&lt;&gt;"",NOT(OR(EXACT(L6,"substantive_difference"),EXACT(L6,"minor_presentation"),EXACT(L6,"version_timing"),EXACT(L6,"non_inconsistency"),EXACT(L6,"indeterminate"))))),"CHECK FIELDS",IF(AND(F6&lt;&gt;"",NOT(OR(EXACT(F6,"no"),EXACT(F6,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F6,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H6" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="I6" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="J6" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="K6" s="8" t="str">
         <f t="shared" si="0"/>
         <v>not_applicable</v>
       </c>
-      <c r="I6" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="J6" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="K6" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="L6" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L6" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M6" s="3"/>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
-      <c r="R6" s="9"/>
+      <c r="R6" s="9" t="s">
+        <v>642</v>
+      </c>
     </row>
     <row r="7" spans="1:18" ht="91.95" customHeight="1">
       <c r="A7" s="1" t="s">
@@ -4098,43 +4204,46 @@
       <c r="C7" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="D7" s="8"/>
+      <c r="D7" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E7" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G7" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A7="",COUNTIF($A$2:$A$8,A7)&lt;&gt;1,LEFT(A7,LEN("2025::jama.2025.19843::"))&lt;&gt;"2025::jama.2025.19843::"),"CHECK KEY",IF(OR(AND(NOT(AND(D7="retain",E7="statistical_results")),H7&lt;&gt;"",NOT(EXACT(H7,"not_applicable"))),AND(NOT(AND(D7="retain",E7="statistical_results")),I7&lt;&gt;"",NOT(EXACT(I7,"not_applicable"))),AND(NOT(AND(D7="retain",E7="statistical_results")),J7&lt;&gt;"",NOT(EXACT(J7,"not_applicable"))),AND(NOT(AND(D7="retain",OR(E7="report_internal_inconsistency",E7="plan_material"))),K7&lt;&gt;"",NOT(EXACT(K7,"not_applicable"))),AND(NOT(AND(D7="retain",E7="protocol_report")),L7&lt;&gt;"",NOT(EXACT(L7,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D7,"retain"),EXACT(D7,"exclude"),EXACT(D7,"discuss"))),NOT(OR(EXACT(E7,"statistical_results"),EXACT(E7,"report_internal_inconsistency"),EXACT(E7,"plan_material"),EXACT(E7,"protocol_report"))),AND(AND(D7="retain",E7="statistical_results"),NOT(OR(EXACT(H7,"confirmed_issue"),EXACT(H7,"probable_issue"),EXACT(H7,"not_issue"),EXACT(H7,"indeterminate")))),AND(AND(D7="retain",E7="statistical_results"),NOT(OR(EXACT(I7,"substantive"),EXACT(I7,"minor_presentation"),EXACT(I7,"indeterminate")))),AND(AND(D7="retain",E7="statistical_results"),J7&lt;&gt;"",NOT(OR(EXACT(J7,"direct"),EXACT(J7,"possible"),EXACT(J7,"unlikely"),EXACT(J7,"unknown")))),AND(AND(D7="retain",OR(E7="report_internal_inconsistency",E7="plan_material")),NOT(OR(EXACT(K7,"substantive_inconsistency"),EXACT(K7,"minor_presentation"),EXACT(K7,"non_inconsistency"),EXACT(K7,"indeterminate")))),AND(AND(D7="retain",E7="protocol_report"),L7&lt;&gt;"",NOT(OR(EXACT(L7,"substantive_difference"),EXACT(L7,"minor_presentation"),EXACT(L7,"version_timing"),EXACT(L7,"non_inconsistency"),EXACT(L7,"indeterminate"))))),"CHECK FIELDS",IF(AND(F7&lt;&gt;"",NOT(OR(EXACT(F7,"no"),EXACT(F7,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F7,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H7" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="I7" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="J7" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="K7" s="8" t="str">
         <f t="shared" si="0"/>
         <v>not_applicable</v>
       </c>
-      <c r="I7" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="J7" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="K7" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="L7" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L7" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M7" s="1"/>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
-      <c r="R7" s="9"/>
+      <c r="R7" s="9" t="s">
+        <v>640</v>
+      </c>
     </row>
     <row r="8" spans="1:18" ht="91.95" customHeight="1">
       <c r="A8" s="3" t="s">
@@ -4146,43 +4255,46 @@
       <c r="C8" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="D8" s="8"/>
+      <c r="D8" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E8" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G8" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A8="",COUNTIF($A$2:$A$8,A8)&lt;&gt;1,LEFT(A8,LEN("2025::jama.2025.19843::"))&lt;&gt;"2025::jama.2025.19843::"),"CHECK KEY",IF(OR(AND(NOT(AND(D8="retain",E8="statistical_results")),H8&lt;&gt;"",NOT(EXACT(H8,"not_applicable"))),AND(NOT(AND(D8="retain",E8="statistical_results")),I8&lt;&gt;"",NOT(EXACT(I8,"not_applicable"))),AND(NOT(AND(D8="retain",E8="statistical_results")),J8&lt;&gt;"",NOT(EXACT(J8,"not_applicable"))),AND(NOT(AND(D8="retain",OR(E8="report_internal_inconsistency",E8="plan_material"))),K8&lt;&gt;"",NOT(EXACT(K8,"not_applicable"))),AND(NOT(AND(D8="retain",E8="protocol_report")),L8&lt;&gt;"",NOT(EXACT(L8,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D8,"retain"),EXACT(D8,"exclude"),EXACT(D8,"discuss"))),NOT(OR(EXACT(E8,"statistical_results"),EXACT(E8,"report_internal_inconsistency"),EXACT(E8,"plan_material"),EXACT(E8,"protocol_report"))),AND(AND(D8="retain",E8="statistical_results"),NOT(OR(EXACT(H8,"confirmed_issue"),EXACT(H8,"probable_issue"),EXACT(H8,"not_issue"),EXACT(H8,"indeterminate")))),AND(AND(D8="retain",E8="statistical_results"),NOT(OR(EXACT(I8,"substantive"),EXACT(I8,"minor_presentation"),EXACT(I8,"indeterminate")))),AND(AND(D8="retain",E8="statistical_results"),J8&lt;&gt;"",NOT(OR(EXACT(J8,"direct"),EXACT(J8,"possible"),EXACT(J8,"unlikely"),EXACT(J8,"unknown")))),AND(AND(D8="retain",OR(E8="report_internal_inconsistency",E8="plan_material")),NOT(OR(EXACT(K8,"substantive_inconsistency"),EXACT(K8,"minor_presentation"),EXACT(K8,"non_inconsistency"),EXACT(K8,"indeterminate")))),AND(AND(D8="retain",E8="protocol_report"),L8&lt;&gt;"",NOT(OR(EXACT(L8,"substantive_difference"),EXACT(L8,"minor_presentation"),EXACT(L8,"version_timing"),EXACT(L8,"non_inconsistency"),EXACT(L8,"indeterminate"))))),"CHECK FIELDS",IF(AND(F8&lt;&gt;"",NOT(OR(EXACT(F8,"no"),EXACT(F8,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F8,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H8" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="I8" s="8" t="str">
+        <f t="shared" si="3"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="J8" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v>not_applicable</v>
+      </c>
+      <c r="K8" s="8" t="str">
         <f t="shared" si="0"/>
         <v>not_applicable</v>
       </c>
-      <c r="I8" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="J8" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="K8" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v>not_applicable</v>
-      </c>
-      <c r="L8" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L8" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M8" s="3"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
-      <c r="R8" s="9"/>
+      <c r="R8" s="9" t="s">
+        <v>638</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:R8" xr:uid="{00000000-0009-0000-0000-00000A000000}"/>
@@ -8824,7 +8936,7 @@
       </c>
       <c r="B4" s="6">
         <f>COUNTIF('C_jama.2024.24764'!$G$2:$G$6,"PRIMARY READY")+COUNTIF('C_jama.2024.27643'!$G$2:$G$17,"PRIMARY READY")+COUNTIF('C_jama.2025.11178'!$G$2:$G$19,"PRIMARY READY")+COUNTIF('C_jama.2025.15185'!$G$2:$G$7,"PRIMARY READY")+COUNTIF('C_jama.2025.15440'!$G$2:$G$2,"PRIMARY READY")+COUNTIF('C_jama.2025.16450'!$G$2:$G$7,"PRIMARY READY")+COUNTIF('C_jama.2025.19563'!$G$2:$G$14,"PRIMARY READY")+COUNTIF('C_jama.2025.19843'!$G$2:$G$8,"PRIMARY READY")+COUNTIF('C_jama.2025.20765'!$G$2:$G$20,"PRIMARY READY")+COUNTIF('C_jama.2025.24175'!$G$2:$G$15,"PRIMARY READY")+COUNTIF('C_jama.2025.4390'!$G$2:$G$14,"PRIMARY READY")+COUNTIF('C_jama.2025.7583'!$G$2:$G$5,"PRIMARY READY")+COUNTIF('C_jama.2025.7710'!$G$2:$G$4,"PRIMARY READY")+COUNTIF('C_jama.2025.9110'!$G$2:$G$4,"PRIMARY READY")+COUNTIF('C_jama.2025.9663'!$G$2:$G$6,"PRIMARY READY")</f>
-        <v>52</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="55.05" customHeight="1">
@@ -8842,7 +8954,7 @@
       </c>
       <c r="B6" s="6">
         <f>B3-B4</f>
-        <v>81</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="55.05" customHeight="1">
@@ -12052,15 +12164,15 @@
         <v>PRIMARY READY</v>
       </c>
       <c r="H2" s="8" t="str">
-        <f t="shared" ref="H2:H7" si="0">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
+        <f t="shared" ref="H2:H6" si="0">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="I2" s="8" t="str">
-        <f t="shared" ref="I2:I7" si="1">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
+        <f t="shared" ref="I2:I6" si="1">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="J2" s="9" t="str">
-        <f t="shared" ref="J2:J7" si="2">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
+        <f t="shared" ref="J2:J6" si="2">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="K2" s="8" t="str">
@@ -12220,7 +12332,7 @@
         <v>520</v>
       </c>
       <c r="L5" s="9" t="str">
-        <f t="shared" ref="L2:L7" si="4">IF(AND(OR(D5="retain",D5=""),E5="protocol_report"),"","not_applicable")</f>
+        <f t="shared" ref="L5:L7" si="4">IF(AND(OR(D5="retain",D5=""),E5="protocol_report"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="M5" s="1"/>

</xml_diff>

<commit_message>
continued updates on 2026-10-21-0532pm
</commit_message>
<xml_diff>
--- a/human_adjudication/human_adjudication_v_2_4_1/2025/human_adjudication_v_2_4_1_2025_R_B.xlsx
+++ b/human_adjudication/human_adjudication_v_2_4_1/2025/human_adjudication_v_2_4_1_2025_R_B.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\bulun-debian\ai-paper-val\human_adjudication\human_adjudication_v_2_4_1\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B834C5-6C0B-4E1D-A8D5-DF7652FE51A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBD5782D-5E8E-448E-8770-ACDB4C786168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="967" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="967" firstSheet="10" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Setup" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1369" uniqueCount="644">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1413" uniqueCount="657">
   <si>
     <t>Field</t>
   </si>
@@ -2081,6 +2081,45 @@
   </si>
   <si>
     <t>SAP §3.6 (Supp2 p.8, OCR) analyzes left ventricular function at day 30 with a Global Net Benefit hierarchical composite (death, heart transplant, LVEF &gt;30%) with bootstrap CI; the report gives only median LVEF among survivors, 45 vs 40%, difference 5 (-0 to 10) (eTable 3, Supp3 p.5). Protocol lists LVEF at day 30 without the composite.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Report (main pp.1, 3): 134 messages = 100 in month 1 (3-4/day), 30 in month 2 (1/day), then 1/month for 4 months. Protocol v6.0 (Supp1 p.53, OCR) states 134 messages but a schedule of 4-5/day for 2 months, 1-2/day for 2 months and 1/week for 2 months (implying well over 300); v4.0 (p.16) states 178 with a similar schedule. The SAP (p.80) matches the report. </t>
+  </si>
+  <si>
+    <t>SAP §'Adjusted analyses' (Supp1 p.92, OCR) plans a fully adjusted model including tobacco use form with education, smoking duration and other baseline characteristics; the report's adjusted RR 3.2 (2.2-5.2) uses covariates 'selected post hoc' (age, sex, education, occupation, smoking duration), without tobacco form (main pp.3-4, Table 2 note a). Disclosed as post hoc.</t>
+  </si>
+  <si>
+    <t>eTable 9 (Supp2 p.13) treatment failure 0.1% vs 0.6% with absolute difference +0.5 (-0.4 to 1.3); mHealth minus usual care is -0.5. Same sign reversal in main Table 2 (p.6) for death (3.5 vs 7.5; printed +4, 1.0 to 7.1) and treatment failure (0.1 vs 0.5; printed +0.4), whereas other rows are mHealth minus usual care.</t>
+  </si>
+  <si>
+    <t>Protocol v6.0 §21.3-21.4 (Supp1 p.49, rendered) includes people who smoke daily OR stopped/reduced since TB diagnosis, excludes retreatment TB and current tobacco pharmacotherapy; report (main p.2) requires daily smoking (&gt;=1 puff on &gt;=25 days last month), omits retreatment, and Figure 1 (p.4) excludes 236 who 'cannot read and no one in home can read SMS', a criterion not in the plan list.</t>
+  </si>
+  <si>
+    <t>Planned primary outcome uses CO &lt;10 ppm (SAP p.84); the CO &lt;6 ppm analysis is described as post hoc sensitivity (main p.3) but its ITT and PP rows sit under the 'Primary outcome' heading of Table 2 (p.6). Labeling issue; the text makes the status clear.</t>
+  </si>
+  <si>
+    <t>eTable 6 (Supp2 p.9): control site 2008 deaths 5 (7.5%); with 40 recruited per cluster (eTable 5 p.8), 5/40 = 12.5%. The count is right: control-site deaths sum to 27 and mHealth to 25, matching Figure 1.</t>
+  </si>
+  <si>
+    <t>Report (main p.3): quit date set 5 days after enrollment, and continuous abstinence is counted from it. The supplied SMS schedule (Supp1 pp.101-103, OCR) sets the quit date 7 days after day 2 (Q(-8) at Tx(+1), i.e., about day 9) and promises 'up to 5' messages/day. The 5-day quit date appears in the protocol only for the Phase 4 face-to-face arm.</t>
+  </si>
+  <si>
+    <t>Protocol v6.0/v4.0 §28.2.2/§11.2.2 (Supp1 pp.66, 28; OCR) plan primary analysis 'in a missing-at-random architecture'; the SAP (p.91) and report (main p.3) treat missing primary outcomes as not abstinent (Russell Standard), with complete-case analysis as sensitivity.</t>
+  </si>
+  <si>
+    <t>Plan (protocol pp.8, 47; SAP p.84; OCR): cotinine by Accutest NicAlert strips, level &lt;3 (100-200 ng/mL) = abstinent. Report (main p.3): a rapid test cassette (AllTest) with 'a negative result' = abstinent; no cutoff given. Device differs and the equivalence of thresholds cannot be checked.</t>
+  </si>
+  <si>
+    <t>eTable 4 (Supp2 p.6), usual care column: drug user 1 (7.4%) and severe pneumonia 1 (7.4%); 1/27 = 3.7%. Also small rounding slips: 16/27 = 59.3% (printed 59.2), 8/52 = 15.4% (15.2), 3/52 = 5.8% (5.7).</t>
+  </si>
+  <si>
+    <t>Protocol v6.0 §28.2.2 (Supp1 p.66; v4.0 p.28; OCR) plans GLMMs with log link and Poisson distribution to estimate RRs; the report (main p.3) uses mixed-effects logistic regression, as does the SAP (p.91-92). Report follows the SAP, not the protocol.</t>
+  </si>
+  <si>
+    <t>SAP subgroup analyses (Supp1 pp.92-93, OCR) include gender (male vs female); the report's prespecified subgroup list (main p.3) and eTable 8 (Supp2 p.12) omit sex and add an ability-to-read-SMS subgroup. No reason given (only 37 women enrolled).</t>
+  </si>
+  <si>
+    <t>Protocol v6.0 Phase 3 sample-size section (Supp1 p.63; OCR) randomizes 27 clusters 18:9, but the power paragraph (p.65) and overview (p.48) still describe 90% power for 16 clusters vs 8 (the v4.0 allocation; change log p.77 records 16/8 -&gt; 18/9).</t>
   </si>
 </sst>
 </file>
@@ -3189,15 +3228,15 @@
         <v>PRIMARY READY</v>
       </c>
       <c r="H2" s="8" t="str">
-        <f t="shared" ref="H2:H14" si="0">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
+        <f t="shared" ref="H2:H11" si="0">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="I2" s="8" t="str">
-        <f t="shared" ref="I2:I14" si="1">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
+        <f t="shared" ref="I2:I11" si="1">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="J2" s="9" t="str">
-        <f t="shared" ref="J2:J14" si="2">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
+        <f t="shared" ref="J2:J11" si="2">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="K2" s="8" t="str">
@@ -3358,7 +3397,7 @@
         <v>not_applicable</v>
       </c>
       <c r="L5" s="9" t="str">
-        <f t="shared" ref="L2:L14" si="4">IF(AND(OR(D5="retain",D5=""),E5="protocol_report"),"","not_applicable")</f>
+        <f t="shared" ref="L5:L14" si="4">IF(AND(OR(D5="retain",D5=""),E5="protocol_report"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="M5" s="1"/>
@@ -3979,7 +4018,7 @@
         <v>not_applicable</v>
       </c>
       <c r="L2" s="9" t="str">
-        <f t="shared" ref="L2:L8" si="1">IF(AND(OR(D2="retain",D2=""),E2="protocol_report"),"","not_applicable")</f>
+        <f t="shared" ref="L2" si="1">IF(AND(OR(D2="retain",D2=""),E2="protocol_report"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="M2" s="3"/>
@@ -4015,15 +4054,15 @@
         <v>PRIMARY READY</v>
       </c>
       <c r="H3" s="8" t="str">
-        <f t="shared" ref="H2:H8" si="2">IF(AND(OR(D3="retain",D3=""),E3="statistical_results"),"","not_applicable")</f>
+        <f t="shared" ref="H3:H8" si="2">IF(AND(OR(D3="retain",D3=""),E3="statistical_results"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="I3" s="8" t="str">
-        <f t="shared" ref="I2:I8" si="3">IF(AND(OR(D3="retain",D3=""),E3="statistical_results"),"","not_applicable")</f>
+        <f t="shared" ref="I3:I8" si="3">IF(AND(OR(D3="retain",D3=""),E3="statistical_results"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="J3" s="9" t="str">
-        <f t="shared" ref="J2:J8" si="4">IF(AND(OR(D3="retain",D3=""),E3="statistical_results"),"","not_applicable")</f>
+        <f t="shared" ref="J3:J8" si="4">IF(AND(OR(D3="retain",D3=""),E3="statistical_results"),"","not_applicable")</f>
         <v>not_applicable</v>
       </c>
       <c r="K3" s="8" t="str">
@@ -4425,16 +4464,18 @@
       <c r="C2" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="D2" s="8"/>
+      <c r="D2" s="8" t="s">
+        <v>488</v>
+      </c>
       <c r="E2" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G2" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A2="",COUNTIF($A$2:$A$20,A2)&lt;&gt;1,LEFT(A2,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D2="retain",E2="statistical_results")),H2&lt;&gt;"",NOT(EXACT(H2,"not_applicable"))),AND(NOT(AND(D2="retain",E2="statistical_results")),I2&lt;&gt;"",NOT(EXACT(I2,"not_applicable"))),AND(NOT(AND(D2="retain",E2="statistical_results")),J2&lt;&gt;"",NOT(EXACT(J2,"not_applicable"))),AND(NOT(AND(D2="retain",OR(E2="report_internal_inconsistency",E2="plan_material"))),K2&lt;&gt;"",NOT(EXACT(K2,"not_applicable"))),AND(NOT(AND(D2="retain",E2="protocol_report")),L2&lt;&gt;"",NOT(EXACT(L2,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D2,"retain"),EXACT(D2,"exclude"),EXACT(D2,"discuss"))),NOT(OR(EXACT(E2,"statistical_results"),EXACT(E2,"report_internal_inconsistency"),EXACT(E2,"plan_material"),EXACT(E2,"protocol_report"))),AND(AND(D2="retain",E2="statistical_results"),NOT(OR(EXACT(H2,"confirmed_issue"),EXACT(H2,"probable_issue"),EXACT(H2,"not_issue"),EXACT(H2,"indeterminate")))),AND(AND(D2="retain",E2="statistical_results"),NOT(OR(EXACT(I2,"substantive"),EXACT(I2,"minor_presentation"),EXACT(I2,"indeterminate")))),AND(AND(D2="retain",E2="statistical_results"),J2&lt;&gt;"",NOT(OR(EXACT(J2,"direct"),EXACT(J2,"possible"),EXACT(J2,"unlikely"),EXACT(J2,"unknown")))),AND(AND(D2="retain",OR(E2="report_internal_inconsistency",E2="plan_material")),NOT(OR(EXACT(K2,"substantive_inconsistency"),EXACT(K2,"minor_presentation"),EXACT(K2,"non_inconsistency"),EXACT(K2,"indeterminate")))),AND(AND(D2="retain",E2="protocol_report"),L2&lt;&gt;"",NOT(OR(EXACT(L2,"substantive_difference"),EXACT(L2,"minor_presentation"),EXACT(L2,"version_timing"),EXACT(L2,"non_inconsistency"),EXACT(L2,"indeterminate"))))),"CHECK FIELDS",IF(AND(F2&lt;&gt;"",NOT(OR(EXACT(F2,"no"),EXACT(F2,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F2,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H2" s="8" t="str">
         <f t="shared" ref="H2:H20" si="0">IF(AND(OR(D2="retain",D2=""),E2="statistical_results"),"","not_applicable")</f>
@@ -4454,14 +4495,16 @@
       </c>
       <c r="L2" s="9" t="str">
         <f t="shared" ref="L2:L20" si="4">IF(AND(OR(D2="retain",D2=""),E2="protocol_report"),"","not_applicable")</f>
-        <v/>
+        <v>not_applicable</v>
       </c>
       <c r="M2" s="3"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
-      <c r="R2" s="9"/>
+      <c r="R2" s="9" t="s">
+        <v>644</v>
+      </c>
     </row>
     <row r="3" spans="1:18" ht="91.95" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -4473,16 +4516,18 @@
       <c r="C3" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="D3" s="8"/>
+      <c r="D3" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E3" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G3" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A3="",COUNTIF($A$2:$A$20,A3)&lt;&gt;1,LEFT(A3,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D3="retain",E3="statistical_results")),H3&lt;&gt;"",NOT(EXACT(H3,"not_applicable"))),AND(NOT(AND(D3="retain",E3="statistical_results")),I3&lt;&gt;"",NOT(EXACT(I3,"not_applicable"))),AND(NOT(AND(D3="retain",E3="statistical_results")),J3&lt;&gt;"",NOT(EXACT(J3,"not_applicable"))),AND(NOT(AND(D3="retain",OR(E3="report_internal_inconsistency",E3="plan_material"))),K3&lt;&gt;"",NOT(EXACT(K3,"not_applicable"))),AND(NOT(AND(D3="retain",E3="protocol_report")),L3&lt;&gt;"",NOT(EXACT(L3,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D3,"retain"),EXACT(D3,"exclude"),EXACT(D3,"discuss"))),NOT(OR(EXACT(E3,"statistical_results"),EXACT(E3,"report_internal_inconsistency"),EXACT(E3,"plan_material"),EXACT(E3,"protocol_report"))),AND(AND(D3="retain",E3="statistical_results"),NOT(OR(EXACT(H3,"confirmed_issue"),EXACT(H3,"probable_issue"),EXACT(H3,"not_issue"),EXACT(H3,"indeterminate")))),AND(AND(D3="retain",E3="statistical_results"),NOT(OR(EXACT(I3,"substantive"),EXACT(I3,"minor_presentation"),EXACT(I3,"indeterminate")))),AND(AND(D3="retain",E3="statistical_results"),J3&lt;&gt;"",NOT(OR(EXACT(J3,"direct"),EXACT(J3,"possible"),EXACT(J3,"unlikely"),EXACT(J3,"unknown")))),AND(AND(D3="retain",OR(E3="report_internal_inconsistency",E3="plan_material")),NOT(OR(EXACT(K3,"substantive_inconsistency"),EXACT(K3,"minor_presentation"),EXACT(K3,"non_inconsistency"),EXACT(K3,"indeterminate")))),AND(AND(D3="retain",E3="protocol_report"),L3&lt;&gt;"",NOT(OR(EXACT(L3,"substantive_difference"),EXACT(L3,"minor_presentation"),EXACT(L3,"version_timing"),EXACT(L3,"non_inconsistency"),EXACT(L3,"indeterminate"))))),"CHECK FIELDS",IF(AND(F3&lt;&gt;"",NOT(OR(EXACT(F3,"no"),EXACT(F3,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F3,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H3" s="8" t="str">
         <f t="shared" si="0"/>
@@ -4500,16 +4545,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L3" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L3" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M3" s="1"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="9"/>
+      <c r="R3" s="9" t="s">
+        <v>647</v>
+      </c>
     </row>
     <row r="4" spans="1:18" ht="91.95" customHeight="1">
       <c r="A4" s="3" t="s">
@@ -4521,16 +4567,18 @@
       <c r="C4" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="D4" s="8"/>
+      <c r="D4" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E4" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G4" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A4="",COUNTIF($A$2:$A$20,A4)&lt;&gt;1,LEFT(A4,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D4="retain",E4="statistical_results")),H4&lt;&gt;"",NOT(EXACT(H4,"not_applicable"))),AND(NOT(AND(D4="retain",E4="statistical_results")),I4&lt;&gt;"",NOT(EXACT(I4,"not_applicable"))),AND(NOT(AND(D4="retain",E4="statistical_results")),J4&lt;&gt;"",NOT(EXACT(J4,"not_applicable"))),AND(NOT(AND(D4="retain",OR(E4="report_internal_inconsistency",E4="plan_material"))),K4&lt;&gt;"",NOT(EXACT(K4,"not_applicable"))),AND(NOT(AND(D4="retain",E4="protocol_report")),L4&lt;&gt;"",NOT(EXACT(L4,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D4,"retain"),EXACT(D4,"exclude"),EXACT(D4,"discuss"))),NOT(OR(EXACT(E4,"statistical_results"),EXACT(E4,"report_internal_inconsistency"),EXACT(E4,"plan_material"),EXACT(E4,"protocol_report"))),AND(AND(D4="retain",E4="statistical_results"),NOT(OR(EXACT(H4,"confirmed_issue"),EXACT(H4,"probable_issue"),EXACT(H4,"not_issue"),EXACT(H4,"indeterminate")))),AND(AND(D4="retain",E4="statistical_results"),NOT(OR(EXACT(I4,"substantive"),EXACT(I4,"minor_presentation"),EXACT(I4,"indeterminate")))),AND(AND(D4="retain",E4="statistical_results"),J4&lt;&gt;"",NOT(OR(EXACT(J4,"direct"),EXACT(J4,"possible"),EXACT(J4,"unlikely"),EXACT(J4,"unknown")))),AND(AND(D4="retain",OR(E4="report_internal_inconsistency",E4="plan_material")),NOT(OR(EXACT(K4,"substantive_inconsistency"),EXACT(K4,"minor_presentation"),EXACT(K4,"non_inconsistency"),EXACT(K4,"indeterminate")))),AND(AND(D4="retain",E4="protocol_report"),L4&lt;&gt;"",NOT(OR(EXACT(L4,"substantive_difference"),EXACT(L4,"minor_presentation"),EXACT(L4,"version_timing"),EXACT(L4,"non_inconsistency"),EXACT(L4,"indeterminate"))))),"CHECK FIELDS",IF(AND(F4&lt;&gt;"",NOT(OR(EXACT(F4,"no"),EXACT(F4,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F4,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H4" s="8" t="str">
         <f t="shared" si="0"/>
@@ -4548,16 +4596,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L4" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L4" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M4" s="3"/>
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
-      <c r="R4" s="9"/>
+      <c r="R4" s="9" t="s">
+        <v>650</v>
+      </c>
     </row>
     <row r="5" spans="1:18" ht="91.95" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -4569,16 +4618,18 @@
       <c r="C5" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="D5" s="8"/>
+      <c r="D5" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E5" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G5" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A5="",COUNTIF($A$2:$A$20,A5)&lt;&gt;1,LEFT(A5,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D5="retain",E5="statistical_results")),H5&lt;&gt;"",NOT(EXACT(H5,"not_applicable"))),AND(NOT(AND(D5="retain",E5="statistical_results")),I5&lt;&gt;"",NOT(EXACT(I5,"not_applicable"))),AND(NOT(AND(D5="retain",E5="statistical_results")),J5&lt;&gt;"",NOT(EXACT(J5,"not_applicable"))),AND(NOT(AND(D5="retain",OR(E5="report_internal_inconsistency",E5="plan_material"))),K5&lt;&gt;"",NOT(EXACT(K5,"not_applicable"))),AND(NOT(AND(D5="retain",E5="protocol_report")),L5&lt;&gt;"",NOT(EXACT(L5,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D5,"retain"),EXACT(D5,"exclude"),EXACT(D5,"discuss"))),NOT(OR(EXACT(E5,"statistical_results"),EXACT(E5,"report_internal_inconsistency"),EXACT(E5,"plan_material"),EXACT(E5,"protocol_report"))),AND(AND(D5="retain",E5="statistical_results"),NOT(OR(EXACT(H5,"confirmed_issue"),EXACT(H5,"probable_issue"),EXACT(H5,"not_issue"),EXACT(H5,"indeterminate")))),AND(AND(D5="retain",E5="statistical_results"),NOT(OR(EXACT(I5,"substantive"),EXACT(I5,"minor_presentation"),EXACT(I5,"indeterminate")))),AND(AND(D5="retain",E5="statistical_results"),J5&lt;&gt;"",NOT(OR(EXACT(J5,"direct"),EXACT(J5,"possible"),EXACT(J5,"unlikely"),EXACT(J5,"unknown")))),AND(AND(D5="retain",OR(E5="report_internal_inconsistency",E5="plan_material")),NOT(OR(EXACT(K5,"substantive_inconsistency"),EXACT(K5,"minor_presentation"),EXACT(K5,"non_inconsistency"),EXACT(K5,"indeterminate")))),AND(AND(D5="retain",E5="protocol_report"),L5&lt;&gt;"",NOT(OR(EXACT(L5,"substantive_difference"),EXACT(L5,"minor_presentation"),EXACT(L5,"version_timing"),EXACT(L5,"non_inconsistency"),EXACT(L5,"indeterminate"))))),"CHECK FIELDS",IF(AND(F5&lt;&gt;"",NOT(OR(EXACT(F5,"no"),EXACT(F5,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F5,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H5" s="8" t="str">
         <f t="shared" si="0"/>
@@ -4596,16 +4647,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L5" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L5" s="9" t="s">
+        <v>518</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
-      <c r="R5" s="9"/>
+      <c r="R5" s="9" t="s">
+        <v>652</v>
+      </c>
     </row>
     <row r="6" spans="1:18" ht="91.95" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -4617,16 +4669,18 @@
       <c r="C6" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="D6" s="8"/>
+      <c r="D6" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E6" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G6" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A6="",COUNTIF($A$2:$A$20,A6)&lt;&gt;1,LEFT(A6,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D6="retain",E6="statistical_results")),H6&lt;&gt;"",NOT(EXACT(H6,"not_applicable"))),AND(NOT(AND(D6="retain",E6="statistical_results")),I6&lt;&gt;"",NOT(EXACT(I6,"not_applicable"))),AND(NOT(AND(D6="retain",E6="statistical_results")),J6&lt;&gt;"",NOT(EXACT(J6,"not_applicable"))),AND(NOT(AND(D6="retain",OR(E6="report_internal_inconsistency",E6="plan_material"))),K6&lt;&gt;"",NOT(EXACT(K6,"not_applicable"))),AND(NOT(AND(D6="retain",E6="protocol_report")),L6&lt;&gt;"",NOT(EXACT(L6,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D6,"retain"),EXACT(D6,"exclude"),EXACT(D6,"discuss"))),NOT(OR(EXACT(E6,"statistical_results"),EXACT(E6,"report_internal_inconsistency"),EXACT(E6,"plan_material"),EXACT(E6,"protocol_report"))),AND(AND(D6="retain",E6="statistical_results"),NOT(OR(EXACT(H6,"confirmed_issue"),EXACT(H6,"probable_issue"),EXACT(H6,"not_issue"),EXACT(H6,"indeterminate")))),AND(AND(D6="retain",E6="statistical_results"),NOT(OR(EXACT(I6,"substantive"),EXACT(I6,"minor_presentation"),EXACT(I6,"indeterminate")))),AND(AND(D6="retain",E6="statistical_results"),J6&lt;&gt;"",NOT(OR(EXACT(J6,"direct"),EXACT(J6,"possible"),EXACT(J6,"unlikely"),EXACT(J6,"unknown")))),AND(AND(D6="retain",OR(E6="report_internal_inconsistency",E6="plan_material")),NOT(OR(EXACT(K6,"substantive_inconsistency"),EXACT(K6,"minor_presentation"),EXACT(K6,"non_inconsistency"),EXACT(K6,"indeterminate")))),AND(AND(D6="retain",E6="protocol_report"),L6&lt;&gt;"",NOT(OR(EXACT(L6,"substantive_difference"),EXACT(L6,"minor_presentation"),EXACT(L6,"version_timing"),EXACT(L6,"non_inconsistency"),EXACT(L6,"indeterminate"))))),"CHECK FIELDS",IF(AND(F6&lt;&gt;"",NOT(OR(EXACT(F6,"no"),EXACT(F6,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F6,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H6" s="8" t="str">
         <f t="shared" si="0"/>
@@ -4644,16 +4698,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L6" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L6" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M6" s="3"/>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
-      <c r="R6" s="9"/>
+      <c r="R6" s="9" t="s">
+        <v>654</v>
+      </c>
     </row>
     <row r="7" spans="1:18" ht="91.95" customHeight="1">
       <c r="A7" s="1" t="s">
@@ -4713,16 +4768,18 @@
       <c r="C8" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="D8" s="8"/>
+      <c r="D8" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E8" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G8" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A8="",COUNTIF($A$2:$A$20,A8)&lt;&gt;1,LEFT(A8,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D8="retain",E8="statistical_results")),H8&lt;&gt;"",NOT(EXACT(H8,"not_applicable"))),AND(NOT(AND(D8="retain",E8="statistical_results")),I8&lt;&gt;"",NOT(EXACT(I8,"not_applicable"))),AND(NOT(AND(D8="retain",E8="statistical_results")),J8&lt;&gt;"",NOT(EXACT(J8,"not_applicable"))),AND(NOT(AND(D8="retain",OR(E8="report_internal_inconsistency",E8="plan_material"))),K8&lt;&gt;"",NOT(EXACT(K8,"not_applicable"))),AND(NOT(AND(D8="retain",E8="protocol_report")),L8&lt;&gt;"",NOT(EXACT(L8,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D8,"retain"),EXACT(D8,"exclude"),EXACT(D8,"discuss"))),NOT(OR(EXACT(E8,"statistical_results"),EXACT(E8,"report_internal_inconsistency"),EXACT(E8,"plan_material"),EXACT(E8,"protocol_report"))),AND(AND(D8="retain",E8="statistical_results"),NOT(OR(EXACT(H8,"confirmed_issue"),EXACT(H8,"probable_issue"),EXACT(H8,"not_issue"),EXACT(H8,"indeterminate")))),AND(AND(D8="retain",E8="statistical_results"),NOT(OR(EXACT(I8,"substantive"),EXACT(I8,"minor_presentation"),EXACT(I8,"indeterminate")))),AND(AND(D8="retain",E8="statistical_results"),J8&lt;&gt;"",NOT(OR(EXACT(J8,"direct"),EXACT(J8,"possible"),EXACT(J8,"unlikely"),EXACT(J8,"unknown")))),AND(AND(D8="retain",OR(E8="report_internal_inconsistency",E8="plan_material")),NOT(OR(EXACT(K8,"substantive_inconsistency"),EXACT(K8,"minor_presentation"),EXACT(K8,"non_inconsistency"),EXACT(K8,"indeterminate")))),AND(AND(D8="retain",E8="protocol_report"),L8&lt;&gt;"",NOT(OR(EXACT(L8,"substantive_difference"),EXACT(L8,"minor_presentation"),EXACT(L8,"version_timing"),EXACT(L8,"non_inconsistency"),EXACT(L8,"indeterminate"))))),"CHECK FIELDS",IF(AND(F8&lt;&gt;"",NOT(OR(EXACT(F8,"no"),EXACT(F8,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F8,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H8" s="8" t="str">
         <f t="shared" si="0"/>
@@ -4740,16 +4797,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L8" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L8" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M8" s="3"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
-      <c r="R8" s="9"/>
+      <c r="R8" s="9" t="s">
+        <v>645</v>
+      </c>
     </row>
     <row r="9" spans="1:18" ht="91.95" customHeight="1">
       <c r="A9" s="1" t="s">
@@ -4761,16 +4819,18 @@
       <c r="C9" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="D9" s="8"/>
+      <c r="D9" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E9" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G9" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A9="",COUNTIF($A$2:$A$20,A9)&lt;&gt;1,LEFT(A9,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D9="retain",E9="statistical_results")),H9&lt;&gt;"",NOT(EXACT(H9,"not_applicable"))),AND(NOT(AND(D9="retain",E9="statistical_results")),I9&lt;&gt;"",NOT(EXACT(I9,"not_applicable"))),AND(NOT(AND(D9="retain",E9="statistical_results")),J9&lt;&gt;"",NOT(EXACT(J9,"not_applicable"))),AND(NOT(AND(D9="retain",OR(E9="report_internal_inconsistency",E9="plan_material"))),K9&lt;&gt;"",NOT(EXACT(K9,"not_applicable"))),AND(NOT(AND(D9="retain",E9="protocol_report")),L9&lt;&gt;"",NOT(EXACT(L9,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D9,"retain"),EXACT(D9,"exclude"),EXACT(D9,"discuss"))),NOT(OR(EXACT(E9,"statistical_results"),EXACT(E9,"report_internal_inconsistency"),EXACT(E9,"plan_material"),EXACT(E9,"protocol_report"))),AND(AND(D9="retain",E9="statistical_results"),NOT(OR(EXACT(H9,"confirmed_issue"),EXACT(H9,"probable_issue"),EXACT(H9,"not_issue"),EXACT(H9,"indeterminate")))),AND(AND(D9="retain",E9="statistical_results"),NOT(OR(EXACT(I9,"substantive"),EXACT(I9,"minor_presentation"),EXACT(I9,"indeterminate")))),AND(AND(D9="retain",E9="statistical_results"),J9&lt;&gt;"",NOT(OR(EXACT(J9,"direct"),EXACT(J9,"possible"),EXACT(J9,"unlikely"),EXACT(J9,"unknown")))),AND(AND(D9="retain",OR(E9="report_internal_inconsistency",E9="plan_material")),NOT(OR(EXACT(K9,"substantive_inconsistency"),EXACT(K9,"minor_presentation"),EXACT(K9,"non_inconsistency"),EXACT(K9,"indeterminate")))),AND(AND(D9="retain",E9="protocol_report"),L9&lt;&gt;"",NOT(OR(EXACT(L9,"substantive_difference"),EXACT(L9,"minor_presentation"),EXACT(L9,"version_timing"),EXACT(L9,"non_inconsistency"),EXACT(L9,"indeterminate"))))),"CHECK FIELDS",IF(AND(F9&lt;&gt;"",NOT(OR(EXACT(F9,"no"),EXACT(F9,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F9,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H9" s="8" t="str">
         <f t="shared" si="0"/>
@@ -4788,16 +4848,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L9" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L9" s="9" t="s">
+        <v>526</v>
       </c>
       <c r="M9" s="1"/>
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
-      <c r="R9" s="9"/>
+      <c r="R9" s="9" t="s">
+        <v>648</v>
+      </c>
     </row>
     <row r="10" spans="1:18" ht="91.95" customHeight="1">
       <c r="A10" s="3" t="s">
@@ -4809,16 +4870,18 @@
       <c r="C10" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="D10" s="8"/>
+      <c r="D10" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E10" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G10" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A10="",COUNTIF($A$2:$A$20,A10)&lt;&gt;1,LEFT(A10,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D10="retain",E10="statistical_results")),H10&lt;&gt;"",NOT(EXACT(H10,"not_applicable"))),AND(NOT(AND(D10="retain",E10="statistical_results")),I10&lt;&gt;"",NOT(EXACT(I10,"not_applicable"))),AND(NOT(AND(D10="retain",E10="statistical_results")),J10&lt;&gt;"",NOT(EXACT(J10,"not_applicable"))),AND(NOT(AND(D10="retain",OR(E10="report_internal_inconsistency",E10="plan_material"))),K10&lt;&gt;"",NOT(EXACT(K10,"not_applicable"))),AND(NOT(AND(D10="retain",E10="protocol_report")),L10&lt;&gt;"",NOT(EXACT(L10,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D10,"retain"),EXACT(D10,"exclude"),EXACT(D10,"discuss"))),NOT(OR(EXACT(E10,"statistical_results"),EXACT(E10,"report_internal_inconsistency"),EXACT(E10,"plan_material"),EXACT(E10,"protocol_report"))),AND(AND(D10="retain",E10="statistical_results"),NOT(OR(EXACT(H10,"confirmed_issue"),EXACT(H10,"probable_issue"),EXACT(H10,"not_issue"),EXACT(H10,"indeterminate")))),AND(AND(D10="retain",E10="statistical_results"),NOT(OR(EXACT(I10,"substantive"),EXACT(I10,"minor_presentation"),EXACT(I10,"indeterminate")))),AND(AND(D10="retain",E10="statistical_results"),J10&lt;&gt;"",NOT(OR(EXACT(J10,"direct"),EXACT(J10,"possible"),EXACT(J10,"unlikely"),EXACT(J10,"unknown")))),AND(AND(D10="retain",OR(E10="report_internal_inconsistency",E10="plan_material")),NOT(OR(EXACT(K10,"substantive_inconsistency"),EXACT(K10,"minor_presentation"),EXACT(K10,"non_inconsistency"),EXACT(K10,"indeterminate")))),AND(AND(D10="retain",E10="protocol_report"),L10&lt;&gt;"",NOT(OR(EXACT(L10,"substantive_difference"),EXACT(L10,"minor_presentation"),EXACT(L10,"version_timing"),EXACT(L10,"non_inconsistency"),EXACT(L10,"indeterminate"))))),"CHECK FIELDS",IF(AND(F10&lt;&gt;"",NOT(OR(EXACT(F10,"no"),EXACT(F10,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F10,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H10" s="8" t="str">
         <f t="shared" si="0"/>
@@ -4836,16 +4899,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L10" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L10" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M10" s="3"/>
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
-      <c r="R10" s="9"/>
+      <c r="R10" s="9" t="s">
+        <v>651</v>
+      </c>
     </row>
     <row r="11" spans="1:18" ht="91.95" customHeight="1">
       <c r="A11" s="1" t="s">
@@ -4857,16 +4921,18 @@
       <c r="C11" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="D11" s="8"/>
+      <c r="D11" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E11" s="8" t="s">
         <v>71</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G11" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A11="",COUNTIF($A$2:$A$20,A11)&lt;&gt;1,LEFT(A11,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D11="retain",E11="statistical_results")),H11&lt;&gt;"",NOT(EXACT(H11,"not_applicable"))),AND(NOT(AND(D11="retain",E11="statistical_results")),I11&lt;&gt;"",NOT(EXACT(I11,"not_applicable"))),AND(NOT(AND(D11="retain",E11="statistical_results")),J11&lt;&gt;"",NOT(EXACT(J11,"not_applicable"))),AND(NOT(AND(D11="retain",OR(E11="report_internal_inconsistency",E11="plan_material"))),K11&lt;&gt;"",NOT(EXACT(K11,"not_applicable"))),AND(NOT(AND(D11="retain",E11="protocol_report")),L11&lt;&gt;"",NOT(EXACT(L11,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D11,"retain"),EXACT(D11,"exclude"),EXACT(D11,"discuss"))),NOT(OR(EXACT(E11,"statistical_results"),EXACT(E11,"report_internal_inconsistency"),EXACT(E11,"plan_material"),EXACT(E11,"protocol_report"))),AND(AND(D11="retain",E11="statistical_results"),NOT(OR(EXACT(H11,"confirmed_issue"),EXACT(H11,"probable_issue"),EXACT(H11,"not_issue"),EXACT(H11,"indeterminate")))),AND(AND(D11="retain",E11="statistical_results"),NOT(OR(EXACT(I11,"substantive"),EXACT(I11,"minor_presentation"),EXACT(I11,"indeterminate")))),AND(AND(D11="retain",E11="statistical_results"),J11&lt;&gt;"",NOT(OR(EXACT(J11,"direct"),EXACT(J11,"possible"),EXACT(J11,"unlikely"),EXACT(J11,"unknown")))),AND(AND(D11="retain",OR(E11="report_internal_inconsistency",E11="plan_material")),NOT(OR(EXACT(K11,"substantive_inconsistency"),EXACT(K11,"minor_presentation"),EXACT(K11,"non_inconsistency"),EXACT(K11,"indeterminate")))),AND(AND(D11="retain",E11="protocol_report"),L11&lt;&gt;"",NOT(OR(EXACT(L11,"substantive_difference"),EXACT(L11,"minor_presentation"),EXACT(L11,"version_timing"),EXACT(L11,"non_inconsistency"),EXACT(L11,"indeterminate"))))),"CHECK FIELDS",IF(AND(F11&lt;&gt;"",NOT(OR(EXACT(F11,"no"),EXACT(F11,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F11,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H11" s="8" t="str">
         <f t="shared" si="0"/>
@@ -4884,16 +4950,17 @@
         <f t="shared" si="3"/>
         <v>not_applicable</v>
       </c>
-      <c r="L11" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="L11" s="9" t="s">
+        <v>554</v>
       </c>
       <c r="M11" s="1"/>
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
-      <c r="R11" s="9"/>
+      <c r="R11" s="9" t="s">
+        <v>655</v>
+      </c>
     </row>
     <row r="12" spans="1:18" ht="91.95" customHeight="1">
       <c r="A12" s="3" t="s">
@@ -5145,16 +5212,18 @@
       <c r="C17" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="D17" s="8"/>
+      <c r="D17" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E17" s="8" t="s">
         <v>81</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G17" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A17="",COUNTIF($A$2:$A$20,A17)&lt;&gt;1,LEFT(A17,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D17="retain",E17="statistical_results")),H17&lt;&gt;"",NOT(EXACT(H17,"not_applicable"))),AND(NOT(AND(D17="retain",E17="statistical_results")),I17&lt;&gt;"",NOT(EXACT(I17,"not_applicable"))),AND(NOT(AND(D17="retain",E17="statistical_results")),J17&lt;&gt;"",NOT(EXACT(J17,"not_applicable"))),AND(NOT(AND(D17="retain",OR(E17="report_internal_inconsistency",E17="plan_material"))),K17&lt;&gt;"",NOT(EXACT(K17,"not_applicable"))),AND(NOT(AND(D17="retain",E17="protocol_report")),L17&lt;&gt;"",NOT(EXACT(L17,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D17,"retain"),EXACT(D17,"exclude"),EXACT(D17,"discuss"))),NOT(OR(EXACT(E17,"statistical_results"),EXACT(E17,"report_internal_inconsistency"),EXACT(E17,"plan_material"),EXACT(E17,"protocol_report"))),AND(AND(D17="retain",E17="statistical_results"),NOT(OR(EXACT(H17,"confirmed_issue"),EXACT(H17,"probable_issue"),EXACT(H17,"not_issue"),EXACT(H17,"indeterminate")))),AND(AND(D17="retain",E17="statistical_results"),NOT(OR(EXACT(I17,"substantive"),EXACT(I17,"minor_presentation"),EXACT(I17,"indeterminate")))),AND(AND(D17="retain",E17="statistical_results"),J17&lt;&gt;"",NOT(OR(EXACT(J17,"direct"),EXACT(J17,"possible"),EXACT(J17,"unlikely"),EXACT(J17,"unknown")))),AND(AND(D17="retain",OR(E17="report_internal_inconsistency",E17="plan_material")),NOT(OR(EXACT(K17,"substantive_inconsistency"),EXACT(K17,"minor_presentation"),EXACT(K17,"non_inconsistency"),EXACT(K17,"indeterminate")))),AND(AND(D17="retain",E17="protocol_report"),L17&lt;&gt;"",NOT(OR(EXACT(L17,"substantive_difference"),EXACT(L17,"minor_presentation"),EXACT(L17,"version_timing"),EXACT(L17,"non_inconsistency"),EXACT(L17,"indeterminate"))))),"CHECK FIELDS",IF(AND(F17&lt;&gt;"",NOT(OR(EXACT(F17,"no"),EXACT(F17,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F17,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
+        <v>PRIMARY READY</v>
       </c>
       <c r="H17" s="8" t="str">
         <f t="shared" si="0"/>
@@ -5168,9 +5237,8 @@
         <f t="shared" si="2"/>
         <v>not_applicable</v>
       </c>
-      <c r="K17" s="8" t="str">
-        <f t="shared" si="3"/>
-        <v/>
+      <c r="K17" s="8" t="s">
+        <v>526</v>
       </c>
       <c r="L17" s="9" t="str">
         <f t="shared" si="4"/>
@@ -5181,7 +5249,9 @@
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
-      <c r="R17" s="9"/>
+      <c r="R17" s="9" t="s">
+        <v>656</v>
+      </c>
     </row>
     <row r="18" spans="1:18" ht="91.95" customHeight="1">
       <c r="A18" s="3" t="s">
@@ -5193,28 +5263,27 @@
       <c r="C18" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="D18" s="8"/>
+      <c r="D18" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E18" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G18" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A18="",COUNTIF($A$2:$A$20,A18)&lt;&gt;1,LEFT(A18,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D18="retain",E18="statistical_results")),H18&lt;&gt;"",NOT(EXACT(H18,"not_applicable"))),AND(NOT(AND(D18="retain",E18="statistical_results")),I18&lt;&gt;"",NOT(EXACT(I18,"not_applicable"))),AND(NOT(AND(D18="retain",E18="statistical_results")),J18&lt;&gt;"",NOT(EXACT(J18,"not_applicable"))),AND(NOT(AND(D18="retain",OR(E18="report_internal_inconsistency",E18="plan_material"))),K18&lt;&gt;"",NOT(EXACT(K18,"not_applicable"))),AND(NOT(AND(D18="retain",E18="protocol_report")),L18&lt;&gt;"",NOT(EXACT(L18,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D18,"retain"),EXACT(D18,"exclude"),EXACT(D18,"discuss"))),NOT(OR(EXACT(E18,"statistical_results"),EXACT(E18,"report_internal_inconsistency"),EXACT(E18,"plan_material"),EXACT(E18,"protocol_report"))),AND(AND(D18="retain",E18="statistical_results"),NOT(OR(EXACT(H18,"confirmed_issue"),EXACT(H18,"probable_issue"),EXACT(H18,"not_issue"),EXACT(H18,"indeterminate")))),AND(AND(D18="retain",E18="statistical_results"),NOT(OR(EXACT(I18,"substantive"),EXACT(I18,"minor_presentation"),EXACT(I18,"indeterminate")))),AND(AND(D18="retain",E18="statistical_results"),J18&lt;&gt;"",NOT(OR(EXACT(J18,"direct"),EXACT(J18,"possible"),EXACT(J18,"unlikely"),EXACT(J18,"unknown")))),AND(AND(D18="retain",OR(E18="report_internal_inconsistency",E18="plan_material")),NOT(OR(EXACT(K18,"substantive_inconsistency"),EXACT(K18,"minor_presentation"),EXACT(K18,"non_inconsistency"),EXACT(K18,"indeterminate")))),AND(AND(D18="retain",E18="protocol_report"),L18&lt;&gt;"",NOT(OR(EXACT(L18,"substantive_difference"),EXACT(L18,"minor_presentation"),EXACT(L18,"version_timing"),EXACT(L18,"non_inconsistency"),EXACT(L18,"indeterminate"))))),"CHECK FIELDS",IF(AND(F18&lt;&gt;"",NOT(OR(EXACT(F18,"no"),EXACT(F18,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F18,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
-      </c>
-      <c r="H18" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I18" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J18" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+        <v>PRIMARY READY</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>536</v>
       </c>
       <c r="K18" s="8" t="str">
         <f t="shared" si="3"/>
@@ -5229,7 +5298,9 @@
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
-      <c r="R18" s="9"/>
+      <c r="R18" s="9" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="19" spans="1:18" ht="91.95" customHeight="1">
       <c r="A19" s="1" t="s">
@@ -5241,28 +5312,27 @@
       <c r="C19" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="D19" s="8"/>
+      <c r="D19" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E19" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G19" s="1" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A19="",COUNTIF($A$2:$A$20,A19)&lt;&gt;1,LEFT(A19,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D19="retain",E19="statistical_results")),H19&lt;&gt;"",NOT(EXACT(H19,"not_applicable"))),AND(NOT(AND(D19="retain",E19="statistical_results")),I19&lt;&gt;"",NOT(EXACT(I19,"not_applicable"))),AND(NOT(AND(D19="retain",E19="statistical_results")),J19&lt;&gt;"",NOT(EXACT(J19,"not_applicable"))),AND(NOT(AND(D19="retain",OR(E19="report_internal_inconsistency",E19="plan_material"))),K19&lt;&gt;"",NOT(EXACT(K19,"not_applicable"))),AND(NOT(AND(D19="retain",E19="protocol_report")),L19&lt;&gt;"",NOT(EXACT(L19,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D19,"retain"),EXACT(D19,"exclude"),EXACT(D19,"discuss"))),NOT(OR(EXACT(E19,"statistical_results"),EXACT(E19,"report_internal_inconsistency"),EXACT(E19,"plan_material"),EXACT(E19,"protocol_report"))),AND(AND(D19="retain",E19="statistical_results"),NOT(OR(EXACT(H19,"confirmed_issue"),EXACT(H19,"probable_issue"),EXACT(H19,"not_issue"),EXACT(H19,"indeterminate")))),AND(AND(D19="retain",E19="statistical_results"),NOT(OR(EXACT(I19,"substantive"),EXACT(I19,"minor_presentation"),EXACT(I19,"indeterminate")))),AND(AND(D19="retain",E19="statistical_results"),J19&lt;&gt;"",NOT(OR(EXACT(J19,"direct"),EXACT(J19,"possible"),EXACT(J19,"unlikely"),EXACT(J19,"unknown")))),AND(AND(D19="retain",OR(E19="report_internal_inconsistency",E19="plan_material")),NOT(OR(EXACT(K19,"substantive_inconsistency"),EXACT(K19,"minor_presentation"),EXACT(K19,"non_inconsistency"),EXACT(K19,"indeterminate")))),AND(AND(D19="retain",E19="protocol_report"),L19&lt;&gt;"",NOT(OR(EXACT(L19,"substantive_difference"),EXACT(L19,"minor_presentation"),EXACT(L19,"version_timing"),EXACT(L19,"non_inconsistency"),EXACT(L19,"indeterminate"))))),"CHECK FIELDS",IF(AND(F19&lt;&gt;"",NOT(OR(EXACT(F19,"no"),EXACT(F19,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F19,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
-      </c>
-      <c r="H19" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I19" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J19" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+        <v>PRIMARY READY</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>526</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>534</v>
       </c>
       <c r="K19" s="8" t="str">
         <f t="shared" si="3"/>
@@ -5277,7 +5347,9 @@
       <c r="O19" s="4"/>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
-      <c r="R19" s="9"/>
+      <c r="R19" s="9" t="s">
+        <v>649</v>
+      </c>
     </row>
     <row r="20" spans="1:18" ht="91.95" customHeight="1">
       <c r="A20" s="3" t="s">
@@ -5289,28 +5361,27 @@
       <c r="C20" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="D20" s="8"/>
+      <c r="D20" s="8" t="s">
+        <v>485</v>
+      </c>
       <c r="E20" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>67</v>
+        <v>570</v>
       </c>
       <c r="G20" s="3" t="str">
         <f>IFERROR(IF(LEN(TRIM(CLEAN(SUBSTITUTE(Setup!$B$2,CHAR(160)," "))))=0,"CHECK REVIEWER ID",IF(OR(A20="",COUNTIF($A$2:$A$20,A20)&lt;&gt;1,LEFT(A20,LEN("2025::jama.2025.20765::"))&lt;&gt;"2025::jama.2025.20765::"),"CHECK KEY",IF(OR(AND(NOT(AND(D20="retain",E20="statistical_results")),H20&lt;&gt;"",NOT(EXACT(H20,"not_applicable"))),AND(NOT(AND(D20="retain",E20="statistical_results")),I20&lt;&gt;"",NOT(EXACT(I20,"not_applicable"))),AND(NOT(AND(D20="retain",E20="statistical_results")),J20&lt;&gt;"",NOT(EXACT(J20,"not_applicable"))),AND(NOT(AND(D20="retain",OR(E20="report_internal_inconsistency",E20="plan_material"))),K20&lt;&gt;"",NOT(EXACT(K20,"not_applicable"))),AND(NOT(AND(D20="retain",E20="protocol_report")),L20&lt;&gt;"",NOT(EXACT(L20,"not_applicable")))),"CLEAR INACTIVE VALUES",IF(OR(NOT(OR(EXACT(D20,"retain"),EXACT(D20,"exclude"),EXACT(D20,"discuss"))),NOT(OR(EXACT(E20,"statistical_results"),EXACT(E20,"report_internal_inconsistency"),EXACT(E20,"plan_material"),EXACT(E20,"protocol_report"))),AND(AND(D20="retain",E20="statistical_results"),NOT(OR(EXACT(H20,"confirmed_issue"),EXACT(H20,"probable_issue"),EXACT(H20,"not_issue"),EXACT(H20,"indeterminate")))),AND(AND(D20="retain",E20="statistical_results"),NOT(OR(EXACT(I20,"substantive"),EXACT(I20,"minor_presentation"),EXACT(I20,"indeterminate")))),AND(AND(D20="retain",E20="statistical_results"),J20&lt;&gt;"",NOT(OR(EXACT(J20,"direct"),EXACT(J20,"possible"),EXACT(J20,"unlikely"),EXACT(J20,"unknown")))),AND(AND(D20="retain",OR(E20="report_internal_inconsistency",E20="plan_material")),NOT(OR(EXACT(K20,"substantive_inconsistency"),EXACT(K20,"minor_presentation"),EXACT(K20,"non_inconsistency"),EXACT(K20,"indeterminate")))),AND(AND(D20="retain",E20="protocol_report"),L20&lt;&gt;"",NOT(OR(EXACT(L20,"substantive_difference"),EXACT(L20,"minor_presentation"),EXACT(L20,"version_timing"),EXACT(L20,"non_inconsistency"),EXACT(L20,"indeterminate"))))),"CHECK FIELDS",IF(AND(F20&lt;&gt;"",NOT(OR(EXACT(F20,"no"),EXACT(F20,"primary_done")))),"CHECK COMPLETE",IF(EXACT(F20,"primary_done"),"PRIMARY READY","PRIMARY DRAFT")))))),"CHECK INPUT / KEY")</f>
-        <v>CHECK FIELDS</v>
-      </c>
-      <c r="H20" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I20" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="J20" s="9" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+        <v>PRIMARY READY</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="I20" s="8" t="s">
+        <v>524</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>534</v>
       </c>
       <c r="K20" s="8" t="str">
         <f t="shared" si="3"/>
@@ -5325,7 +5396,9 @@
       <c r="O20" s="4"/>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
-      <c r="R20" s="9"/>
+      <c r="R20" s="9" t="s">
+        <v>646</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:R20" xr:uid="{00000000-0009-0000-0000-00000B000000}"/>
@@ -8936,7 +9009,7 @@
       </c>
       <c r="B4" s="6">
         <f>COUNTIF('C_jama.2024.24764'!$G$2:$G$6,"PRIMARY READY")+COUNTIF('C_jama.2024.27643'!$G$2:$G$17,"PRIMARY READY")+COUNTIF('C_jama.2025.11178'!$G$2:$G$19,"PRIMARY READY")+COUNTIF('C_jama.2025.15185'!$G$2:$G$7,"PRIMARY READY")+COUNTIF('C_jama.2025.15440'!$G$2:$G$2,"PRIMARY READY")+COUNTIF('C_jama.2025.16450'!$G$2:$G$7,"PRIMARY READY")+COUNTIF('C_jama.2025.19563'!$G$2:$G$14,"PRIMARY READY")+COUNTIF('C_jama.2025.19843'!$G$2:$G$8,"PRIMARY READY")+COUNTIF('C_jama.2025.20765'!$G$2:$G$20,"PRIMARY READY")+COUNTIF('C_jama.2025.24175'!$G$2:$G$15,"PRIMARY READY")+COUNTIF('C_jama.2025.4390'!$G$2:$G$14,"PRIMARY READY")+COUNTIF('C_jama.2025.7583'!$G$2:$G$5,"PRIMARY READY")+COUNTIF('C_jama.2025.7710'!$G$2:$G$4,"PRIMARY READY")+COUNTIF('C_jama.2025.9110'!$G$2:$G$4,"PRIMARY READY")+COUNTIF('C_jama.2025.9663'!$G$2:$G$6,"PRIMARY READY")</f>
-        <v>72</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="55.05" customHeight="1">
@@ -8954,7 +9027,7 @@
       </c>
       <c r="B6" s="6">
         <f>B3-B4</f>
-        <v>61</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="55.05" customHeight="1">

</xml_diff>